<commit_message>
exploration system 2 and new BGM
</commit_message>
<xml_diff>
--- a/context/card_data_demo.xlsx
+++ b/context/card_data_demo.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1429">
   <si>
     <t>Table 1</t>
   </si>
@@ -247,7 +247,7 @@
     <t>Pit Lord</t>
   </si>
   <si>
-    <t>his card is destroyed if battle with Divine Unit. After this card attacked, halve its ATK&amp;DEF permanently</t>
+    <t>This card is destroyed if battle with Divine Unit. After this card attacked, halve its ATK&amp;DEF permanently</t>
   </si>
   <si>
     <t>Ancient Lich</t>
@@ -316,7 +316,7 @@
     <t>Leech Man</t>
   </si>
   <si>
-    <t>+20 DEF permanently each time it performed attack and survive. With mutagen flag : +45 ATK</t>
+    <t>+10 DEF permanently after it performed attack on unit. Also +10 ATK with mutagen flag</t>
   </si>
   <si>
     <t>Immortal Vampire</t>
@@ -403,7 +403,7 @@
     <t>Mafia Associates</t>
   </si>
   <si>
-    <t>If this card is exposed, its defense becomes 0</t>
+    <t>At the end of the turn that it’s been exposed, its defense becomes 0</t>
   </si>
   <si>
     <t>Silver Dragon</t>
@@ -535,7 +535,7 @@
     <t>Sniping Fairy</t>
   </si>
   <si>
-    <t>-20 ATK if exposed</t>
+    <t>At the end of the turn that it’s been exposed, -20 ATK</t>
   </si>
   <si>
     <t>Bomber Fairy</t>
@@ -664,7 +664,7 @@
     <t>Mephisto the Fallen</t>
   </si>
   <si>
-    <t>After this card attacked successfully, its ATK becomes 0 permanently</t>
+    <t>After this card attacked unit successfully, its ATK becomes 0 permanently</t>
   </si>
   <si>
     <t>Joseph the Battle Priest</t>
@@ -760,7 +760,7 @@
     <t>Cursed Well</t>
   </si>
   <si>
-    <t>+15 ATK if exposed</t>
+    <t>At the end of the turn that it’s been exposed, +15 ATK</t>
   </si>
   <si>
     <t>Shredder Doll</t>
@@ -1093,7 +1093,7 @@
     <t>Armored Monkey</t>
   </si>
   <si>
-    <t>+10 ATK if there is face-up Nature card</t>
+    <t>+10 ATK if there is another face-up Nature card</t>
   </si>
   <si>
     <t>Magical Butterfly</t>
@@ -1462,7 +1462,7 @@
     <t>Blue Mage</t>
   </si>
   <si>
-    <t>If this card battles non-Arcane card, flip a coins. If both are head, destroy it.</t>
+    <t>If this card battles non-Arcane card, flip two coins. If both are head, destroy it.</t>
   </si>
   <si>
     <t>Spell Sniper</t>
@@ -2321,10 +2321,10 @@
     <t>Diamond Unicorn</t>
   </si>
   <si>
-    <t>+15 ATK until ????</t>
-  </si>
-  <si>
-    <t>+15 ATK until the end of this turn, once.</t>
+    <t>Once Union, ??? until this turn’s end</t>
+  </si>
+  <si>
+    <t>Once Union, +15 ATK until this turn’s end</t>
   </si>
   <si>
     <t>1 ??? + 1 ??? + 500 cost</t>
@@ -3454,6 +3454,21 @@
     <t>Nanomites Dragon</t>
   </si>
   <si>
+    <t>Capnomancer</t>
+  </si>
+  <si>
+    <t>At the start of your turn, you can destroy this card to ???</t>
+  </si>
+  <si>
+    <t>At the start of your turn, you can destroy this card to revive Pyromancer</t>
+  </si>
+  <si>
+    <t>1 ???</t>
+  </si>
+  <si>
+    <t>1 Pyromancer + 1000 cost</t>
+  </si>
+  <si>
     <t>Booster Pack - Blightsilver / 9</t>
   </si>
   <si>
@@ -3788,7 +3803,7 @@
     <t>Alarm</t>
   </si>
   <si>
-    <t>Unil the end of this urn, All face-up Anima monster gain +10 DEF</t>
+    <t>Until the end of this urn, All face-up Anima monster gain +10 DEF</t>
   </si>
   <si>
     <t>Protective Instinct</t>
@@ -3819,6 +3834,12 @@
   </si>
   <si>
     <t>If you have 1500 or less crystal, drain crystal from foe until both players have same amount of crystals</t>
+  </si>
+  <si>
+    <t>Tripwire</t>
+  </si>
+  <si>
+    <t>Destroy the attacker with 20 or less ATK. Attacker side pay no cost.</t>
   </si>
   <si>
     <t>Illustration</t>
@@ -7683,7 +7704,7 @@
       <c r="O37" s="10"/>
       <c r="P37" s="10"/>
     </row>
-    <row r="38" ht="56.05" customHeight="1">
+    <row r="38" ht="44.05" customHeight="1">
       <c r="A38" t="s" s="8">
         <v>98</v>
       </c>
@@ -8392,7 +8413,7 @@
       <c r="O54" s="10"/>
       <c r="P54" s="10"/>
     </row>
-    <row r="55" ht="32.05" customHeight="1">
+    <row r="55" ht="44.05" customHeight="1">
       <c r="A55" t="s" s="8">
         <v>127</v>
       </c>
@@ -8461,7 +8482,9 @@
         <v>130</v>
       </c>
       <c r="I56" s="10"/>
-      <c r="J56" s="10"/>
+      <c r="J56" t="s" s="17">
+        <v>35</v>
+      </c>
       <c r="K56" s="16">
         <f>(D56*6)+(E56*4)</f>
         <v>1280</v>
@@ -8498,7 +8521,9 @@
         <v>39</v>
       </c>
       <c r="I57" s="10"/>
-      <c r="J57" s="10"/>
+      <c r="J57" t="s" s="17">
+        <v>35</v>
+      </c>
       <c r="K57" s="16">
         <f>(D57*6)+(E57*4)</f>
         <v>160</v>
@@ -8535,7 +8560,9 @@
         <v>39</v>
       </c>
       <c r="I58" s="10"/>
-      <c r="J58" s="10"/>
+      <c r="J58" t="s" s="17">
+        <v>35</v>
+      </c>
       <c r="K58" s="16">
         <f>(D58*6)+(E58*4)</f>
         <v>140</v>
@@ -9506,7 +9533,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="83" ht="20.05" customHeight="1">
+    <row r="83" ht="32.05" customHeight="1">
       <c r="A83" t="s" s="8">
         <v>171</v>
       </c>
@@ -11095,7 +11122,7 @@
       <c r="O123" s="10"/>
       <c r="P123" s="10"/>
     </row>
-    <row r="124" ht="20.05" customHeight="1">
+    <row r="124" ht="32.05" customHeight="1">
       <c r="A124" t="s" s="8">
         <v>246</v>
       </c>
@@ -16596,10 +16623,10 @@
         <v>800</v>
       </c>
       <c r="D266" s="16">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="E266" s="16">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="F266" t="s" s="17">
         <v>7</v>
@@ -16616,7 +16643,7 @@
       </c>
       <c r="K266" s="16">
         <f>(D266*6)+(E266*4)</f>
-        <v>450</v>
+        <v>350</v>
       </c>
       <c r="L266" t="s" s="17">
         <v>35</v>
@@ -25213,7 +25240,7 @@
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="16">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="E19" s="16">
         <v>35</v>
@@ -26601,7 +26628,7 @@
       </c>
       <c r="C55" s="10"/>
       <c r="D55" s="16">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="E55" s="16">
         <v>40</v>
@@ -27655,19 +27682,41 @@
       <c r="N85" s="10"/>
       <c r="O85" s="10"/>
     </row>
-    <row r="86" ht="20.05" customHeight="1">
-      <c r="A86" s="11"/>
-      <c r="B86" s="12"/>
-      <c r="C86" s="10"/>
-      <c r="D86" s="10"/>
-      <c r="E86" s="10"/>
-      <c r="F86" s="10"/>
+    <row r="86" ht="80.05" customHeight="1">
+      <c r="A86" t="s" s="8">
+        <v>1044</v>
+      </c>
+      <c r="B86" t="s" s="9">
+        <v>663</v>
+      </c>
+      <c r="C86" s="16">
+        <v>0</v>
+      </c>
+      <c r="D86" s="16">
+        <v>0</v>
+      </c>
+      <c r="E86" s="16">
+        <v>120</v>
+      </c>
+      <c r="F86" t="s" s="17">
+        <v>7</v>
+      </c>
       <c r="G86" s="10"/>
-      <c r="H86" s="10"/>
-      <c r="I86" s="10"/>
-      <c r="J86" s="10"/>
-      <c r="K86" s="10"/>
-      <c r="L86" s="10"/>
+      <c r="H86" t="s" s="17">
+        <v>1045</v>
+      </c>
+      <c r="I86" t="s" s="17">
+        <v>1046</v>
+      </c>
+      <c r="J86" t="s" s="17">
+        <v>1047</v>
+      </c>
+      <c r="K86" t="s" s="17">
+        <v>1048</v>
+      </c>
+      <c r="L86" t="s" s="17">
+        <v>971</v>
+      </c>
       <c r="M86" s="10"/>
       <c r="N86" s="10"/>
       <c r="O86" s="10"/>
@@ -35685,23 +35734,23 @@
       </c>
       <c r="N2" t="s" s="3">
         <f>"Booster Pack - Blightsilver / "&amp;COUNTIF(N3:N545,"Yes")</f>
-        <v>1044</v>
+        <v>1049</v>
       </c>
       <c r="O2" t="s" s="3">
         <f>"Booster Pack - Unseen Presence / "&amp;COUNTIF(O3:O545,"Yes")</f>
-        <v>1045</v>
+        <v>1050</v>
       </c>
       <c r="P2" t="s" s="3">
         <f>"Booster Pack - Wind of Dominance / "&amp;COUNTIF(P3:P545,"Yes")</f>
-        <v>1046</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="3" ht="44.25" customHeight="1">
       <c r="A3" t="s" s="5">
-        <v>1047</v>
+        <v>1052</v>
       </c>
       <c r="B3" t="s" s="6">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C3" s="14">
         <v>0</v>
@@ -35713,7 +35762,7 @@
         <v>1</v>
       </c>
       <c r="H3" t="s" s="15">
-        <v>1049</v>
+        <v>1054</v>
       </c>
       <c r="I3" s="7"/>
       <c r="J3" t="s" s="15">
@@ -35732,10 +35781,10 @@
     </row>
     <row r="4" ht="44.05" customHeight="1">
       <c r="A4" t="s" s="8">
-        <v>1050</v>
+        <v>1055</v>
       </c>
       <c r="B4" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C4" s="16">
         <v>200</v>
@@ -35747,7 +35796,7 @@
         <v>2</v>
       </c>
       <c r="H4" t="s" s="17">
-        <v>1051</v>
+        <v>1056</v>
       </c>
       <c r="I4" s="10"/>
       <c r="J4" t="s" s="17">
@@ -35766,10 +35815,10 @@
     </row>
     <row r="5" ht="44.05" customHeight="1">
       <c r="A5" t="s" s="8">
-        <v>1052</v>
+        <v>1057</v>
       </c>
       <c r="B5" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C5" s="16">
         <v>0</v>
@@ -35781,7 +35830,7 @@
         <v>1</v>
       </c>
       <c r="H5" t="s" s="17">
-        <v>1053</v>
+        <v>1058</v>
       </c>
       <c r="I5" s="10"/>
       <c r="J5" t="s" s="17">
@@ -35800,10 +35849,10 @@
     </row>
     <row r="6" ht="44.05" customHeight="1">
       <c r="A6" t="s" s="8">
-        <v>1054</v>
+        <v>1059</v>
       </c>
       <c r="B6" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C6" s="16">
         <v>0</v>
@@ -35815,7 +35864,7 @@
         <v>2</v>
       </c>
       <c r="H6" t="s" s="17">
-        <v>1055</v>
+        <v>1060</v>
       </c>
       <c r="I6" s="10"/>
       <c r="J6" t="s" s="17">
@@ -35834,10 +35883,10 @@
     </row>
     <row r="7" ht="32.05" customHeight="1">
       <c r="A7" t="s" s="8">
-        <v>1056</v>
+        <v>1061</v>
       </c>
       <c r="B7" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C7" s="16">
         <v>500</v>
@@ -35849,7 +35898,7 @@
         <v>3</v>
       </c>
       <c r="H7" t="s" s="17">
-        <v>1057</v>
+        <v>1062</v>
       </c>
       <c r="I7" s="10"/>
       <c r="J7" t="s" s="17">
@@ -35868,10 +35917,10 @@
     </row>
     <row r="8" ht="44.05" customHeight="1">
       <c r="A8" t="s" s="8">
-        <v>1058</v>
+        <v>1063</v>
       </c>
       <c r="B8" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C8" s="16">
         <v>0</v>
@@ -35883,7 +35932,7 @@
         <v>5</v>
       </c>
       <c r="H8" t="s" s="17">
-        <v>1059</v>
+        <v>1064</v>
       </c>
       <c r="I8" s="10"/>
       <c r="J8" t="s" s="17">
@@ -35902,10 +35951,10 @@
     </row>
     <row r="9" ht="32.05" customHeight="1">
       <c r="A9" t="s" s="8">
-        <v>1060</v>
+        <v>1065</v>
       </c>
       <c r="B9" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C9" s="16">
         <v>800</v>
@@ -35917,7 +35966,7 @@
         <v>4</v>
       </c>
       <c r="H9" t="s" s="17">
-        <v>1061</v>
+        <v>1066</v>
       </c>
       <c r="I9" s="10"/>
       <c r="J9" t="s" s="17">
@@ -35936,10 +35985,10 @@
     </row>
     <row r="10" ht="32.05" customHeight="1">
       <c r="A10" t="s" s="8">
-        <v>1062</v>
+        <v>1067</v>
       </c>
       <c r="B10" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C10" s="16">
         <v>250</v>
@@ -35951,7 +36000,7 @@
         <v>2</v>
       </c>
       <c r="H10" t="s" s="17">
-        <v>1063</v>
+        <v>1068</v>
       </c>
       <c r="I10" s="10"/>
       <c r="J10" t="s" s="17">
@@ -35970,10 +36019,10 @@
     </row>
     <row r="11" ht="32.05" customHeight="1">
       <c r="A11" t="s" s="8">
-        <v>1064</v>
+        <v>1069</v>
       </c>
       <c r="B11" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C11" s="16">
         <v>1000</v>
@@ -35985,7 +36034,7 @@
         <v>3</v>
       </c>
       <c r="H11" t="s" s="17">
-        <v>1065</v>
+        <v>1070</v>
       </c>
       <c r="I11" s="10"/>
       <c r="J11" t="s" s="17">
@@ -36004,10 +36053,10 @@
     </row>
     <row r="12" ht="44.05" customHeight="1">
       <c r="A12" t="s" s="8">
-        <v>1066</v>
+        <v>1071</v>
       </c>
       <c r="B12" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C12" s="16">
         <v>200</v>
@@ -36019,7 +36068,7 @@
         <v>2</v>
       </c>
       <c r="H12" t="s" s="17">
-        <v>1067</v>
+        <v>1072</v>
       </c>
       <c r="I12" s="10"/>
       <c r="J12" t="s" s="17">
@@ -36034,10 +36083,10 @@
     </row>
     <row r="13" ht="32.05" customHeight="1">
       <c r="A13" t="s" s="8">
-        <v>1068</v>
+        <v>1073</v>
       </c>
       <c r="B13" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C13" s="16">
         <v>500</v>
@@ -36049,7 +36098,7 @@
         <v>3</v>
       </c>
       <c r="H13" t="s" s="17">
-        <v>1069</v>
+        <v>1074</v>
       </c>
       <c r="I13" s="10"/>
       <c r="J13" t="s" s="17">
@@ -36068,10 +36117,10 @@
     </row>
     <row r="14" ht="20.05" customHeight="1">
       <c r="A14" t="s" s="8">
-        <v>1070</v>
+        <v>1075</v>
       </c>
       <c r="B14" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C14" s="16">
         <v>1500</v>
@@ -36083,7 +36132,7 @@
         <v>5</v>
       </c>
       <c r="H14" t="s" s="17">
-        <v>1071</v>
+        <v>1076</v>
       </c>
       <c r="I14" s="10"/>
       <c r="J14" t="s" s="17">
@@ -36102,10 +36151,10 @@
     </row>
     <row r="15" ht="32.05" customHeight="1">
       <c r="A15" t="s" s="8">
-        <v>1072</v>
+        <v>1077</v>
       </c>
       <c r="B15" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C15" s="16">
         <v>500</v>
@@ -36117,7 +36166,7 @@
         <v>4</v>
       </c>
       <c r="H15" t="s" s="17">
-        <v>1073</v>
+        <v>1078</v>
       </c>
       <c r="I15" s="10"/>
       <c r="J15" t="s" s="17">
@@ -36136,10 +36185,10 @@
     </row>
     <row r="16" ht="32.05" customHeight="1">
       <c r="A16" t="s" s="8">
-        <v>1074</v>
+        <v>1079</v>
       </c>
       <c r="B16" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C16" s="16">
         <v>1500</v>
@@ -36151,7 +36200,7 @@
         <v>5</v>
       </c>
       <c r="H16" t="s" s="17">
-        <v>1075</v>
+        <v>1080</v>
       </c>
       <c r="I16" s="10"/>
       <c r="J16" t="s" s="17">
@@ -36170,10 +36219,10 @@
     </row>
     <row r="17" ht="44.05" customHeight="1">
       <c r="A17" t="s" s="8">
-        <v>1076</v>
+        <v>1081</v>
       </c>
       <c r="B17" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C17" s="16">
         <v>900</v>
@@ -36185,7 +36234,7 @@
         <v>4</v>
       </c>
       <c r="H17" t="s" s="17">
-        <v>1077</v>
+        <v>1082</v>
       </c>
       <c r="I17" s="10"/>
       <c r="J17" t="s" s="17">
@@ -36204,10 +36253,10 @@
     </row>
     <row r="18" ht="44.05" customHeight="1">
       <c r="A18" t="s" s="8">
-        <v>1078</v>
+        <v>1083</v>
       </c>
       <c r="B18" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C18" s="16">
         <v>0</v>
@@ -36219,7 +36268,7 @@
         <v>3</v>
       </c>
       <c r="H18" t="s" s="17">
-        <v>1079</v>
+        <v>1084</v>
       </c>
       <c r="I18" s="10"/>
       <c r="J18" t="s" s="17">
@@ -36238,10 +36287,10 @@
     </row>
     <row r="19" ht="44.05" customHeight="1">
       <c r="A19" t="s" s="8">
-        <v>1080</v>
+        <v>1085</v>
       </c>
       <c r="B19" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C19" s="16">
         <v>800</v>
@@ -36253,7 +36302,7 @@
         <v>4</v>
       </c>
       <c r="H19" t="s" s="17">
-        <v>1081</v>
+        <v>1086</v>
       </c>
       <c r="I19" s="10"/>
       <c r="J19" t="s" s="17">
@@ -36268,10 +36317,10 @@
     </row>
     <row r="20" ht="44.05" customHeight="1">
       <c r="A20" t="s" s="8">
-        <v>1082</v>
+        <v>1087</v>
       </c>
       <c r="B20" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C20" s="16">
         <v>600</v>
@@ -36283,7 +36332,7 @@
         <v>4</v>
       </c>
       <c r="H20" t="s" s="17">
-        <v>1083</v>
+        <v>1088</v>
       </c>
       <c r="I20" s="10"/>
       <c r="J20" t="s" s="17">
@@ -36298,10 +36347,10 @@
     </row>
     <row r="21" ht="44.05" customHeight="1">
       <c r="A21" t="s" s="8">
-        <v>1084</v>
+        <v>1089</v>
       </c>
       <c r="B21" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C21" s="16">
         <v>0</v>
@@ -36313,7 +36362,7 @@
         <v>1</v>
       </c>
       <c r="H21" t="s" s="17">
-        <v>1085</v>
+        <v>1090</v>
       </c>
       <c r="I21" s="10"/>
       <c r="J21" t="s" s="17">
@@ -36332,10 +36381,10 @@
     </row>
     <row r="22" ht="44.05" customHeight="1">
       <c r="A22" t="s" s="8">
-        <v>1086</v>
+        <v>1091</v>
       </c>
       <c r="B22" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C22" s="16">
         <v>50</v>
@@ -36347,7 +36396,7 @@
         <v>2</v>
       </c>
       <c r="H22" t="s" s="17">
-        <v>1087</v>
+        <v>1092</v>
       </c>
       <c r="I22" s="10"/>
       <c r="J22" t="s" s="17">
@@ -36362,10 +36411,10 @@
     </row>
     <row r="23" ht="32.05" customHeight="1">
       <c r="A23" t="s" s="8">
-        <v>1088</v>
+        <v>1093</v>
       </c>
       <c r="B23" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C23" s="16">
         <v>100</v>
@@ -36377,7 +36426,7 @@
         <v>3</v>
       </c>
       <c r="H23" t="s" s="17">
-        <v>1089</v>
+        <v>1094</v>
       </c>
       <c r="I23" s="10"/>
       <c r="J23" t="s" s="17">
@@ -36392,10 +36441,10 @@
     </row>
     <row r="24" ht="44.05" customHeight="1">
       <c r="A24" t="s" s="8">
-        <v>1090</v>
+        <v>1095</v>
       </c>
       <c r="B24" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C24" s="16">
         <v>1000</v>
@@ -36407,7 +36456,7 @@
         <v>5</v>
       </c>
       <c r="H24" t="s" s="17">
-        <v>1091</v>
+        <v>1096</v>
       </c>
       <c r="I24" s="10"/>
       <c r="J24" t="s" s="17">
@@ -36422,10 +36471,10 @@
     </row>
     <row r="25" ht="44.05" customHeight="1">
       <c r="A25" t="s" s="8">
-        <v>1092</v>
+        <v>1097</v>
       </c>
       <c r="B25" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C25" s="16">
         <v>850</v>
@@ -36437,7 +36486,7 @@
         <v>2</v>
       </c>
       <c r="H25" t="s" s="17">
-        <v>1093</v>
+        <v>1098</v>
       </c>
       <c r="I25" s="10"/>
       <c r="J25" t="s" s="17">
@@ -36452,10 +36501,10 @@
     </row>
     <row r="26" ht="32.05" customHeight="1">
       <c r="A26" t="s" s="8">
-        <v>1094</v>
+        <v>1099</v>
       </c>
       <c r="B26" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C26" s="16">
         <v>600</v>
@@ -36467,7 +36516,7 @@
         <v>1</v>
       </c>
       <c r="H26" t="s" s="17">
-        <v>1095</v>
+        <v>1100</v>
       </c>
       <c r="I26" s="10"/>
       <c r="J26" t="s" s="17">
@@ -36482,10 +36531,10 @@
     </row>
     <row r="27" ht="44.05" customHeight="1">
       <c r="A27" t="s" s="8">
-        <v>1096</v>
+        <v>1101</v>
       </c>
       <c r="B27" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C27" s="16">
         <v>600</v>
@@ -36497,7 +36546,7 @@
         <v>1</v>
       </c>
       <c r="H27" t="s" s="17">
-        <v>1097</v>
+        <v>1102</v>
       </c>
       <c r="I27" s="10"/>
       <c r="J27" t="s" s="17">
@@ -36512,10 +36561,10 @@
     </row>
     <row r="28" ht="44.05" customHeight="1">
       <c r="A28" t="s" s="8">
-        <v>1098</v>
+        <v>1103</v>
       </c>
       <c r="B28" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C28" s="16">
         <v>600</v>
@@ -36527,7 +36576,7 @@
         <v>1</v>
       </c>
       <c r="H28" t="s" s="17">
-        <v>1099</v>
+        <v>1104</v>
       </c>
       <c r="I28" s="10"/>
       <c r="J28" t="s" s="17">
@@ -36542,10 +36591,10 @@
     </row>
     <row r="29" ht="32.05" customHeight="1">
       <c r="A29" t="s" s="8">
-        <v>1100</v>
+        <v>1105</v>
       </c>
       <c r="B29" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C29" s="16">
         <v>600</v>
@@ -36557,7 +36606,7 @@
         <v>1</v>
       </c>
       <c r="H29" t="s" s="17">
-        <v>1101</v>
+        <v>1106</v>
       </c>
       <c r="I29" s="10"/>
       <c r="J29" t="s" s="17">
@@ -36572,10 +36621,10 @@
     </row>
     <row r="30" ht="44.05" customHeight="1">
       <c r="A30" t="s" s="8">
-        <v>1102</v>
+        <v>1107</v>
       </c>
       <c r="B30" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C30" s="16">
         <v>600</v>
@@ -36587,7 +36636,7 @@
         <v>1</v>
       </c>
       <c r="H30" t="s" s="17">
-        <v>1103</v>
+        <v>1108</v>
       </c>
       <c r="I30" s="10"/>
       <c r="J30" t="s" s="17">
@@ -36602,10 +36651,10 @@
     </row>
     <row r="31" ht="44.05" customHeight="1">
       <c r="A31" t="s" s="8">
-        <v>1104</v>
+        <v>1109</v>
       </c>
       <c r="B31" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C31" s="16">
         <v>600</v>
@@ -36617,7 +36666,7 @@
         <v>1</v>
       </c>
       <c r="H31" t="s" s="17">
-        <v>1105</v>
+        <v>1110</v>
       </c>
       <c r="I31" s="10"/>
       <c r="J31" t="s" s="17">
@@ -36632,10 +36681,10 @@
     </row>
     <row r="32" ht="44.05" customHeight="1">
       <c r="A32" t="s" s="8">
-        <v>1106</v>
+        <v>1111</v>
       </c>
       <c r="B32" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C32" s="16">
         <v>600</v>
@@ -36647,7 +36696,7 @@
         <v>1</v>
       </c>
       <c r="H32" t="s" s="17">
-        <v>1107</v>
+        <v>1112</v>
       </c>
       <c r="I32" s="10"/>
       <c r="J32" t="s" s="17">
@@ -36662,10 +36711,10 @@
     </row>
     <row r="33" ht="32.05" customHeight="1">
       <c r="A33" t="s" s="8">
-        <v>1108</v>
+        <v>1113</v>
       </c>
       <c r="B33" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C33" s="16">
         <v>300</v>
@@ -36677,7 +36726,7 @@
         <v>2</v>
       </c>
       <c r="H33" t="s" s="17">
-        <v>1109</v>
+        <v>1114</v>
       </c>
       <c r="I33" s="10"/>
       <c r="J33" t="s" s="17">
@@ -36692,10 +36741,10 @@
     </row>
     <row r="34" ht="44.05" customHeight="1">
       <c r="A34" t="s" s="8">
-        <v>1110</v>
+        <v>1115</v>
       </c>
       <c r="B34" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C34" s="16">
         <v>800</v>
@@ -36707,7 +36756,7 @@
         <v>3</v>
       </c>
       <c r="H34" t="s" s="17">
-        <v>1111</v>
+        <v>1116</v>
       </c>
       <c r="I34" s="10"/>
       <c r="J34" t="s" s="17">
@@ -36722,10 +36771,10 @@
     </row>
     <row r="35" ht="56.05" customHeight="1">
       <c r="A35" t="s" s="8">
-        <v>1112</v>
+        <v>1117</v>
       </c>
       <c r="B35" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C35" s="16">
         <v>800</v>
@@ -36737,7 +36786,7 @@
         <v>3</v>
       </c>
       <c r="H35" t="s" s="17">
-        <v>1113</v>
+        <v>1118</v>
       </c>
       <c r="I35" s="10"/>
       <c r="J35" t="s" s="17">
@@ -36752,10 +36801,10 @@
     </row>
     <row r="36" ht="44.05" customHeight="1">
       <c r="A36" t="s" s="8">
-        <v>1114</v>
+        <v>1119</v>
       </c>
       <c r="B36" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C36" s="16">
         <v>800</v>
@@ -36767,7 +36816,7 @@
         <v>3</v>
       </c>
       <c r="H36" t="s" s="17">
-        <v>1115</v>
+        <v>1120</v>
       </c>
       <c r="I36" s="10"/>
       <c r="J36" t="s" s="17">
@@ -36782,10 +36831,10 @@
     </row>
     <row r="37" ht="44.05" customHeight="1">
       <c r="A37" t="s" s="8">
-        <v>1116</v>
+        <v>1121</v>
       </c>
       <c r="B37" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C37" s="16">
         <v>800</v>
@@ -36797,7 +36846,7 @@
         <v>3</v>
       </c>
       <c r="H37" t="s" s="17">
-        <v>1117</v>
+        <v>1122</v>
       </c>
       <c r="I37" s="10"/>
       <c r="J37" t="s" s="17">
@@ -36812,10 +36861,10 @@
     </row>
     <row r="38" ht="44.05" customHeight="1">
       <c r="A38" t="s" s="8">
-        <v>1118</v>
+        <v>1123</v>
       </c>
       <c r="B38" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C38" s="16">
         <v>800</v>
@@ -36827,7 +36876,7 @@
         <v>3</v>
       </c>
       <c r="H38" t="s" s="17">
-        <v>1119</v>
+        <v>1124</v>
       </c>
       <c r="I38" s="10"/>
       <c r="J38" t="s" s="17">
@@ -36842,10 +36891,10 @@
     </row>
     <row r="39" ht="56.05" customHeight="1">
       <c r="A39" t="s" s="8">
-        <v>1120</v>
+        <v>1125</v>
       </c>
       <c r="B39" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C39" s="16">
         <v>800</v>
@@ -36857,7 +36906,7 @@
         <v>3</v>
       </c>
       <c r="H39" t="s" s="17">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="I39" s="10"/>
       <c r="J39" t="s" s="17">
@@ -36872,10 +36921,10 @@
     </row>
     <row r="40" ht="56.05" customHeight="1">
       <c r="A40" t="s" s="8">
-        <v>1122</v>
+        <v>1127</v>
       </c>
       <c r="B40" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C40" s="16">
         <v>800</v>
@@ -36887,7 +36936,7 @@
         <v>3</v>
       </c>
       <c r="H40" t="s" s="17">
-        <v>1123</v>
+        <v>1128</v>
       </c>
       <c r="I40" s="10"/>
       <c r="J40" t="s" s="17">
@@ -36902,10 +36951,10 @@
     </row>
     <row r="41" ht="44.05" customHeight="1">
       <c r="A41" t="s" s="8">
-        <v>1124</v>
+        <v>1129</v>
       </c>
       <c r="B41" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C41" s="16">
         <v>1200</v>
@@ -36917,7 +36966,7 @@
         <v>3</v>
       </c>
       <c r="H41" t="s" s="17">
-        <v>1125</v>
+        <v>1130</v>
       </c>
       <c r="I41" s="10"/>
       <c r="J41" t="s" s="17">
@@ -36932,10 +36981,10 @@
     </row>
     <row r="42" ht="44.05" customHeight="1">
       <c r="A42" t="s" s="8">
-        <v>1126</v>
+        <v>1131</v>
       </c>
       <c r="B42" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C42" s="16">
         <v>1500</v>
@@ -36947,7 +36996,7 @@
         <v>4</v>
       </c>
       <c r="H42" t="s" s="17">
-        <v>1127</v>
+        <v>1132</v>
       </c>
       <c r="I42" s="10"/>
       <c r="J42" t="s" s="17">
@@ -36962,10 +37011,10 @@
     </row>
     <row r="43" ht="44.05" customHeight="1">
       <c r="A43" t="s" s="8">
-        <v>1128</v>
+        <v>1133</v>
       </c>
       <c r="B43" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C43" s="16">
         <v>100</v>
@@ -36977,7 +37026,7 @@
         <v>2</v>
       </c>
       <c r="H43" t="s" s="17">
-        <v>1129</v>
+        <v>1134</v>
       </c>
       <c r="I43" s="10"/>
       <c r="J43" t="s" s="17">
@@ -36996,10 +37045,10 @@
     </row>
     <row r="44" ht="32.05" customHeight="1">
       <c r="A44" t="s" s="8">
-        <v>1130</v>
+        <v>1135</v>
       </c>
       <c r="B44" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C44" s="16">
         <v>700</v>
@@ -37011,7 +37060,7 @@
         <v>1</v>
       </c>
       <c r="H44" t="s" s="17">
-        <v>1131</v>
+        <v>1136</v>
       </c>
       <c r="I44" s="10"/>
       <c r="J44" t="s" s="17">
@@ -37030,10 +37079,10 @@
     </row>
     <row r="45" ht="32.05" customHeight="1">
       <c r="A45" t="s" s="8">
-        <v>1132</v>
+        <v>1137</v>
       </c>
       <c r="B45" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C45" s="16">
         <v>1200</v>
@@ -37045,7 +37094,7 @@
         <v>1</v>
       </c>
       <c r="H45" t="s" s="17">
-        <v>1133</v>
+        <v>1138</v>
       </c>
       <c r="I45" s="10"/>
       <c r="J45" s="10"/>
@@ -37058,10 +37107,10 @@
     </row>
     <row r="46" ht="32.05" customHeight="1">
       <c r="A46" t="s" s="8">
-        <v>1134</v>
+        <v>1139</v>
       </c>
       <c r="B46" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C46" s="16">
         <v>1500</v>
@@ -37073,7 +37122,7 @@
         <v>1</v>
       </c>
       <c r="H46" t="s" s="17">
-        <v>1135</v>
+        <v>1140</v>
       </c>
       <c r="I46" s="10"/>
       <c r="J46" s="10"/>
@@ -37086,10 +37135,10 @@
     </row>
     <row r="47" ht="32.05" customHeight="1">
       <c r="A47" t="s" s="8">
-        <v>1136</v>
+        <v>1141</v>
       </c>
       <c r="B47" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C47" s="16">
         <v>950</v>
@@ -37101,7 +37150,7 @@
         <v>1</v>
       </c>
       <c r="H47" t="s" s="17">
-        <v>1137</v>
+        <v>1142</v>
       </c>
       <c r="I47" s="10"/>
       <c r="J47" s="10"/>
@@ -37114,10 +37163,10 @@
     </row>
     <row r="48" ht="44.05" customHeight="1">
       <c r="A48" t="s" s="8">
-        <v>1138</v>
+        <v>1143</v>
       </c>
       <c r="B48" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C48" s="16">
         <v>0</v>
@@ -37129,7 +37178,7 @@
         <v>3</v>
       </c>
       <c r="H48" t="s" s="17">
-        <v>1139</v>
+        <v>1144</v>
       </c>
       <c r="I48" s="10"/>
       <c r="J48" s="10"/>
@@ -37142,10 +37191,10 @@
     </row>
     <row r="49" ht="68.05" customHeight="1">
       <c r="A49" t="s" s="8">
-        <v>1140</v>
+        <v>1145</v>
       </c>
       <c r="B49" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C49" s="16">
         <v>2000</v>
@@ -37157,7 +37206,7 @@
         <v>5</v>
       </c>
       <c r="H49" t="s" s="17">
-        <v>1141</v>
+        <v>1146</v>
       </c>
       <c r="I49" s="10"/>
       <c r="J49" s="10"/>
@@ -37170,10 +37219,10 @@
     </row>
     <row r="50" ht="44.05" customHeight="1">
       <c r="A50" t="s" s="8">
-        <v>1142</v>
+        <v>1147</v>
       </c>
       <c r="B50" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C50" s="16">
         <v>100</v>
@@ -37185,7 +37234,7 @@
         <v>1</v>
       </c>
       <c r="H50" t="s" s="17">
-        <v>1143</v>
+        <v>1148</v>
       </c>
       <c r="I50" s="10"/>
       <c r="J50" s="10"/>
@@ -37198,7 +37247,7 @@
     </row>
     <row r="51" ht="44.05" customHeight="1">
       <c r="A51" t="s" s="8">
-        <v>1144</v>
+        <v>1149</v>
       </c>
       <c r="B51" s="12"/>
       <c r="C51" s="16">
@@ -37211,7 +37260,7 @@
         <v>1</v>
       </c>
       <c r="H51" t="s" s="17">
-        <v>1145</v>
+        <v>1150</v>
       </c>
       <c r="I51" s="10"/>
       <c r="J51" s="10"/>
@@ -37224,10 +37273,10 @@
     </row>
     <row r="52" ht="32.05" customHeight="1">
       <c r="A52" t="s" s="8">
-        <v>1146</v>
+        <v>1151</v>
       </c>
       <c r="B52" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C52" s="16">
         <v>0</v>
@@ -37239,7 +37288,7 @@
         <v>2</v>
       </c>
       <c r="H52" t="s" s="17">
-        <v>1147</v>
+        <v>1152</v>
       </c>
       <c r="I52" s="10"/>
       <c r="J52" t="s" s="17">
@@ -37258,7 +37307,7 @@
     </row>
     <row r="53" ht="32.05" customHeight="1">
       <c r="A53" t="s" s="8">
-        <v>1148</v>
+        <v>1153</v>
       </c>
       <c r="B53" s="12"/>
       <c r="C53" s="16">
@@ -37271,7 +37320,7 @@
         <v>2</v>
       </c>
       <c r="H53" t="s" s="17">
-        <v>1149</v>
+        <v>1154</v>
       </c>
       <c r="I53" s="10"/>
       <c r="J53" s="10"/>
@@ -37284,7 +37333,7 @@
     </row>
     <row r="54" ht="32.05" customHeight="1">
       <c r="A54" t="s" s="8">
-        <v>1150</v>
+        <v>1155</v>
       </c>
       <c r="B54" s="12"/>
       <c r="C54" s="16">
@@ -37297,7 +37346,7 @@
         <v>3</v>
       </c>
       <c r="H54" t="s" s="17">
-        <v>1151</v>
+        <v>1156</v>
       </c>
       <c r="I54" s="10"/>
       <c r="J54" s="10"/>
@@ -37310,10 +37359,10 @@
     </row>
     <row r="55" ht="32.05" customHeight="1">
       <c r="A55" t="s" s="8">
-        <v>1152</v>
+        <v>1157</v>
       </c>
       <c r="B55" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C55" s="16">
         <v>0</v>
@@ -37325,7 +37374,7 @@
         <v>1</v>
       </c>
       <c r="H55" t="s" s="17">
-        <v>1153</v>
+        <v>1158</v>
       </c>
       <c r="I55" s="10"/>
       <c r="J55" t="s" s="17">
@@ -37344,10 +37393,10 @@
     </row>
     <row r="56" ht="44.05" customHeight="1">
       <c r="A56" t="s" s="8">
-        <v>1154</v>
+        <v>1159</v>
       </c>
       <c r="B56" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C56" s="16">
         <v>0</v>
@@ -37359,7 +37408,7 @@
         <v>1</v>
       </c>
       <c r="H56" t="s" s="17">
-        <v>1155</v>
+        <v>1160</v>
       </c>
       <c r="I56" s="10"/>
       <c r="J56" t="s" s="17">
@@ -37378,7 +37427,7 @@
     </row>
     <row r="57" ht="44.05" customHeight="1">
       <c r="A57" t="s" s="8">
-        <v>1156</v>
+        <v>1161</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="16">
@@ -37391,7 +37440,7 @@
         <v>1</v>
       </c>
       <c r="H57" t="s" s="17">
-        <v>1157</v>
+        <v>1162</v>
       </c>
       <c r="I57" s="10"/>
       <c r="J57" s="10"/>
@@ -37404,10 +37453,10 @@
     </row>
     <row r="58" ht="44.05" customHeight="1">
       <c r="A58" t="s" s="8">
-        <v>1158</v>
+        <v>1163</v>
       </c>
       <c r="B58" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C58" s="16">
         <v>0</v>
@@ -37419,7 +37468,7 @@
         <v>2</v>
       </c>
       <c r="H58" t="s" s="17">
-        <v>1159</v>
+        <v>1164</v>
       </c>
       <c r="I58" s="10"/>
       <c r="J58" t="s" s="17">
@@ -37438,7 +37487,7 @@
     </row>
     <row r="59" ht="44.05" customHeight="1">
       <c r="A59" t="s" s="8">
-        <v>1160</v>
+        <v>1165</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="16">
@@ -37451,7 +37500,7 @@
         <v>2</v>
       </c>
       <c r="H59" t="s" s="17">
-        <v>1161</v>
+        <v>1166</v>
       </c>
       <c r="I59" s="10"/>
       <c r="J59" s="10"/>
@@ -37464,10 +37513,10 @@
     </row>
     <row r="60" ht="56.05" customHeight="1">
       <c r="A60" t="s" s="8">
-        <v>1162</v>
+        <v>1167</v>
       </c>
       <c r="B60" t="s" s="9">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="C60" s="16">
         <v>0</v>
@@ -37479,7 +37528,7 @@
         <v>1</v>
       </c>
       <c r="H60" t="s" s="17">
-        <v>1163</v>
+        <v>1168</v>
       </c>
       <c r="I60" s="10"/>
       <c r="J60" t="s" s="17">
@@ -37498,7 +37547,7 @@
     </row>
     <row r="61" ht="56.05" customHeight="1">
       <c r="A61" t="s" s="8">
-        <v>1164</v>
+        <v>1169</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="16">
@@ -37511,7 +37560,7 @@
         <v>5</v>
       </c>
       <c r="H61" t="s" s="17">
-        <v>1165</v>
+        <v>1170</v>
       </c>
       <c r="I61" s="10"/>
       <c r="J61" s="10"/>
@@ -37522,15 +37571,21 @@
       <c r="O61" s="10"/>
       <c r="P61" s="10"/>
     </row>
-    <row r="62" ht="20.05" customHeight="1">
-      <c r="A62" s="11"/>
+    <row r="62" ht="44.05" customHeight="1">
+      <c r="A62" t="s" s="8">
+        <v>1171</v>
+      </c>
       <c r="B62" s="12"/>
-      <c r="C62" s="10"/>
+      <c r="C62" s="16">
+        <v>300</v>
+      </c>
       <c r="D62" s="10"/>
       <c r="E62" s="10"/>
       <c r="F62" s="10"/>
       <c r="G62" s="10"/>
-      <c r="H62" s="10"/>
+      <c r="H62" t="s" s="17">
+        <v>1172</v>
+      </c>
       <c r="I62" s="10"/>
       <c r="J62" s="10"/>
       <c r="K62" s="10"/>
@@ -46312,7 +46367,7 @@
         <v>24</v>
       </c>
       <c r="J2" t="s" s="3">
-        <v>1166</v>
+        <v>1173</v>
       </c>
       <c r="K2" t="s" s="3">
         <v>26</v>
@@ -46325,23 +46380,23 @@
       </c>
       <c r="N2" t="s" s="3">
         <f>"Booster Pack - Blightsilver / "&amp;COUNTIF(N3:N556,"Yes")</f>
-        <v>1167</v>
+        <v>1174</v>
       </c>
       <c r="O2" t="s" s="3">
         <f>"Booster Pack - Unseen Presence / "&amp;COUNTIF(O3:O556,"Yes")</f>
-        <v>1168</v>
+        <v>1175</v>
       </c>
       <c r="P2" t="s" s="3">
         <f>"Booster Pack - Wind of Dominance / "&amp;COUNTIF(P3:P556,"Yes")</f>
-        <v>1169</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="3" ht="32.25" customHeight="1">
       <c r="A3" t="s" s="5">
-        <v>1170</v>
+        <v>1177</v>
       </c>
       <c r="B3" t="s" s="6">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C3" s="14">
         <v>0</v>
@@ -46353,7 +46408,7 @@
         <v>1</v>
       </c>
       <c r="H3" t="s" s="15">
-        <v>1172</v>
+        <v>1179</v>
       </c>
       <c r="I3" s="7"/>
       <c r="J3" t="s" s="15">
@@ -46368,10 +46423,10 @@
     </row>
     <row r="4" ht="20.05" customHeight="1">
       <c r="A4" t="s" s="8">
-        <v>1173</v>
+        <v>1180</v>
       </c>
       <c r="B4" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C4" s="16">
         <v>0</v>
@@ -46383,7 +46438,7 @@
         <v>1</v>
       </c>
       <c r="H4" t="s" s="17">
-        <v>1174</v>
+        <v>1181</v>
       </c>
       <c r="I4" s="10"/>
       <c r="J4" t="s" s="17">
@@ -46402,10 +46457,10 @@
     </row>
     <row r="5" ht="32.05" customHeight="1">
       <c r="A5" t="s" s="8">
-        <v>1175</v>
+        <v>1182</v>
       </c>
       <c r="B5" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C5" s="16">
         <v>0</v>
@@ -46417,7 +46472,7 @@
         <v>3</v>
       </c>
       <c r="H5" t="s" s="17">
-        <v>1176</v>
+        <v>1183</v>
       </c>
       <c r="I5" s="10"/>
       <c r="J5" t="s" s="17">
@@ -46432,10 +46487,10 @@
     </row>
     <row r="6" ht="80.05" customHeight="1">
       <c r="A6" t="s" s="8">
-        <v>1177</v>
+        <v>1184</v>
       </c>
       <c r="B6" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C6" s="16">
         <v>0</v>
@@ -46447,7 +46502,7 @@
         <v>5</v>
       </c>
       <c r="H6" t="s" s="17">
-        <v>1178</v>
+        <v>1185</v>
       </c>
       <c r="I6" s="10"/>
       <c r="J6" t="s" s="17">
@@ -46462,10 +46517,10 @@
     </row>
     <row r="7" ht="56.05" customHeight="1">
       <c r="A7" t="s" s="8">
-        <v>1179</v>
+        <v>1186</v>
       </c>
       <c r="B7" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C7" s="16">
         <v>0</v>
@@ -46477,7 +46532,7 @@
         <v>2</v>
       </c>
       <c r="H7" t="s" s="17">
-        <v>1180</v>
+        <v>1187</v>
       </c>
       <c r="I7" s="10"/>
       <c r="J7" t="s" s="17">
@@ -46492,10 +46547,10 @@
     </row>
     <row r="8" ht="56.05" customHeight="1">
       <c r="A8" t="s" s="8">
-        <v>1181</v>
+        <v>1188</v>
       </c>
       <c r="B8" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C8" s="16">
         <v>0</v>
@@ -46507,7 +46562,7 @@
         <v>3</v>
       </c>
       <c r="H8" t="s" s="17">
-        <v>1182</v>
+        <v>1189</v>
       </c>
       <c r="I8" s="10"/>
       <c r="J8" t="s" s="17">
@@ -46522,10 +46577,10 @@
     </row>
     <row r="9" ht="56.05" customHeight="1">
       <c r="A9" t="s" s="8">
-        <v>1183</v>
+        <v>1190</v>
       </c>
       <c r="B9" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C9" s="16">
         <v>0</v>
@@ -46537,7 +46592,7 @@
         <v>4</v>
       </c>
       <c r="H9" t="s" s="17">
-        <v>1184</v>
+        <v>1191</v>
       </c>
       <c r="I9" s="10"/>
       <c r="J9" t="s" s="17">
@@ -46552,10 +46607,10 @@
     </row>
     <row r="10" ht="32.05" customHeight="1">
       <c r="A10" t="s" s="8">
-        <v>1185</v>
+        <v>1192</v>
       </c>
       <c r="B10" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C10" s="16">
         <v>0</v>
@@ -46567,7 +46622,7 @@
         <v>2</v>
       </c>
       <c r="H10" t="s" s="17">
-        <v>1186</v>
+        <v>1193</v>
       </c>
       <c r="I10" s="10"/>
       <c r="J10" t="s" s="17">
@@ -46586,10 +46641,10 @@
     </row>
     <row r="11" ht="44.05" customHeight="1">
       <c r="A11" t="s" s="8">
-        <v>1187</v>
+        <v>1194</v>
       </c>
       <c r="B11" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C11" s="16">
         <v>0</v>
@@ -46601,7 +46656,7 @@
         <v>3</v>
       </c>
       <c r="H11" t="s" s="17">
-        <v>1188</v>
+        <v>1195</v>
       </c>
       <c r="I11" s="10"/>
       <c r="J11" t="s" s="17">
@@ -46620,10 +46675,10 @@
     </row>
     <row r="12" ht="44.05" customHeight="1">
       <c r="A12" t="s" s="8">
-        <v>1189</v>
+        <v>1196</v>
       </c>
       <c r="B12" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C12" s="16">
         <v>0</v>
@@ -46635,7 +46690,7 @@
         <v>4</v>
       </c>
       <c r="H12" t="s" s="17">
-        <v>1190</v>
+        <v>1197</v>
       </c>
       <c r="I12" s="10"/>
       <c r="J12" t="s" s="17">
@@ -46654,10 +46709,10 @@
     </row>
     <row r="13" ht="44.05" customHeight="1">
       <c r="A13" t="s" s="8">
-        <v>1191</v>
+        <v>1198</v>
       </c>
       <c r="B13" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C13" s="16">
         <v>0</v>
@@ -46669,7 +46724,7 @@
         <v>4</v>
       </c>
       <c r="H13" t="s" s="17">
-        <v>1192</v>
+        <v>1199</v>
       </c>
       <c r="I13" s="10"/>
       <c r="J13" t="s" s="17">
@@ -46688,10 +46743,10 @@
     </row>
     <row r="14" ht="56.05" customHeight="1">
       <c r="A14" t="s" s="8">
-        <v>1193</v>
+        <v>1200</v>
       </c>
       <c r="B14" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C14" s="16">
         <v>3000</v>
@@ -46703,7 +46758,7 @@
         <v>5</v>
       </c>
       <c r="H14" t="s" s="17">
-        <v>1194</v>
+        <v>1201</v>
       </c>
       <c r="I14" s="10"/>
       <c r="J14" t="s" s="17">
@@ -46718,10 +46773,10 @@
     </row>
     <row r="15" ht="56.05" customHeight="1">
       <c r="A15" t="s" s="8">
-        <v>1195</v>
+        <v>1202</v>
       </c>
       <c r="B15" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C15" s="16">
         <v>2000</v>
@@ -46733,7 +46788,7 @@
         <v>3</v>
       </c>
       <c r="H15" t="s" s="17">
-        <v>1196</v>
+        <v>1203</v>
       </c>
       <c r="I15" s="10"/>
       <c r="J15" t="s" s="17">
@@ -46748,10 +46803,10 @@
     </row>
     <row r="16" ht="32.05" customHeight="1">
       <c r="A16" t="s" s="8">
-        <v>1197</v>
+        <v>1204</v>
       </c>
       <c r="B16" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C16" s="16">
         <v>1000</v>
@@ -46763,7 +46818,7 @@
         <v>4</v>
       </c>
       <c r="H16" t="s" s="17">
-        <v>1198</v>
+        <v>1205</v>
       </c>
       <c r="I16" s="10"/>
       <c r="J16" t="s" s="17">
@@ -46782,10 +46837,10 @@
     </row>
     <row r="17" ht="32.05" customHeight="1">
       <c r="A17" t="s" s="8">
-        <v>1199</v>
+        <v>1206</v>
       </c>
       <c r="B17" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C17" s="16">
         <v>1000</v>
@@ -46797,7 +46852,7 @@
         <v>3</v>
       </c>
       <c r="H17" t="s" s="17">
-        <v>1200</v>
+        <v>1207</v>
       </c>
       <c r="I17" s="10"/>
       <c r="J17" t="s" s="17">
@@ -46816,10 +46871,10 @@
     </row>
     <row r="18" ht="56.05" customHeight="1">
       <c r="A18" t="s" s="8">
-        <v>1201</v>
+        <v>1208</v>
       </c>
       <c r="B18" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C18" s="16">
         <v>500</v>
@@ -46831,7 +46886,7 @@
         <v>2</v>
       </c>
       <c r="H18" t="s" s="17">
-        <v>1202</v>
+        <v>1209</v>
       </c>
       <c r="I18" s="10"/>
       <c r="J18" t="s" s="17">
@@ -46846,10 +46901,10 @@
     </row>
     <row r="19" ht="32.05" customHeight="1">
       <c r="A19" t="s" s="8">
-        <v>1203</v>
+        <v>1210</v>
       </c>
       <c r="B19" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C19" s="16">
         <v>1000</v>
@@ -46861,7 +46916,7 @@
         <v>4</v>
       </c>
       <c r="H19" t="s" s="17">
-        <v>1204</v>
+        <v>1211</v>
       </c>
       <c r="I19" s="10"/>
       <c r="J19" t="s" s="17">
@@ -46876,10 +46931,10 @@
     </row>
     <row r="20" ht="56.05" customHeight="1">
       <c r="A20" t="s" s="8">
-        <v>1205</v>
+        <v>1212</v>
       </c>
       <c r="B20" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C20" s="16">
         <v>600</v>
@@ -46891,7 +46946,7 @@
         <v>3</v>
       </c>
       <c r="H20" t="s" s="17">
-        <v>1206</v>
+        <v>1213</v>
       </c>
       <c r="I20" s="10"/>
       <c r="J20" t="s" s="17">
@@ -46906,10 +46961,10 @@
     </row>
     <row r="21" ht="32.05" customHeight="1">
       <c r="A21" t="s" s="8">
-        <v>1207</v>
+        <v>1214</v>
       </c>
       <c r="B21" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C21" s="16">
         <v>1500</v>
@@ -46921,7 +46976,7 @@
         <v>4</v>
       </c>
       <c r="H21" t="s" s="17">
-        <v>1208</v>
+        <v>1215</v>
       </c>
       <c r="I21" s="10"/>
       <c r="J21" t="s" s="17">
@@ -46936,10 +46991,10 @@
     </row>
     <row r="22" ht="44.05" customHeight="1">
       <c r="A22" t="s" s="8">
-        <v>1209</v>
+        <v>1216</v>
       </c>
       <c r="B22" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C22" s="16">
         <v>850</v>
@@ -46951,7 +47006,7 @@
         <v>3</v>
       </c>
       <c r="H22" t="s" s="17">
-        <v>1210</v>
+        <v>1217</v>
       </c>
       <c r="I22" s="10"/>
       <c r="J22" t="s" s="17">
@@ -46966,10 +47021,10 @@
     </row>
     <row r="23" ht="44.05" customHeight="1">
       <c r="A23" t="s" s="8">
-        <v>1211</v>
+        <v>1218</v>
       </c>
       <c r="B23" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C23" s="16">
         <v>1000</v>
@@ -46981,7 +47036,7 @@
         <v>5</v>
       </c>
       <c r="H23" t="s" s="17">
-        <v>1212</v>
+        <v>1219</v>
       </c>
       <c r="I23" s="10"/>
       <c r="J23" t="s" s="17">
@@ -47000,10 +47055,10 @@
     </row>
     <row r="24" ht="20.05" customHeight="1">
       <c r="A24" t="s" s="8">
-        <v>1213</v>
+        <v>1220</v>
       </c>
       <c r="B24" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C24" s="16">
         <v>2000</v>
@@ -47015,7 +47070,7 @@
         <v>4</v>
       </c>
       <c r="H24" t="s" s="17">
-        <v>1214</v>
+        <v>1221</v>
       </c>
       <c r="I24" s="10"/>
       <c r="J24" t="s" s="17">
@@ -47030,10 +47085,10 @@
     </row>
     <row r="25" ht="56.05" customHeight="1">
       <c r="A25" t="s" s="8">
-        <v>1215</v>
+        <v>1222</v>
       </c>
       <c r="B25" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C25" s="16">
         <v>1000</v>
@@ -47045,7 +47100,7 @@
         <v>3</v>
       </c>
       <c r="H25" t="s" s="17">
-        <v>1216</v>
+        <v>1223</v>
       </c>
       <c r="I25" s="10"/>
       <c r="J25" t="s" s="17">
@@ -47064,10 +47119,10 @@
     </row>
     <row r="26" ht="80.05" customHeight="1">
       <c r="A26" t="s" s="8">
-        <v>1217</v>
+        <v>1224</v>
       </c>
       <c r="B26" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C26" s="16">
         <v>2000</v>
@@ -47079,7 +47134,7 @@
         <v>5</v>
       </c>
       <c r="H26" t="s" s="17">
-        <v>1218</v>
+        <v>1225</v>
       </c>
       <c r="I26" s="10"/>
       <c r="J26" t="s" s="17">
@@ -47094,10 +47149,10 @@
     </row>
     <row r="27" ht="20.05" customHeight="1">
       <c r="A27" t="s" s="8">
-        <v>1219</v>
+        <v>1226</v>
       </c>
       <c r="B27" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C27" s="16">
         <v>600</v>
@@ -47109,7 +47164,7 @@
         <v>1</v>
       </c>
       <c r="H27" t="s" s="17">
-        <v>1220</v>
+        <v>1227</v>
       </c>
       <c r="I27" s="10"/>
       <c r="J27" t="s" s="17">
@@ -47128,10 +47183,10 @@
     </row>
     <row r="28" ht="44.05" customHeight="1">
       <c r="A28" t="s" s="8">
-        <v>1221</v>
+        <v>1228</v>
       </c>
       <c r="B28" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C28" s="16">
         <v>500</v>
@@ -47143,7 +47198,7 @@
         <v>2</v>
       </c>
       <c r="H28" t="s" s="17">
-        <v>1222</v>
+        <v>1229</v>
       </c>
       <c r="I28" s="10"/>
       <c r="J28" t="s" s="17">
@@ -47158,10 +47213,10 @@
     </row>
     <row r="29" ht="80.05" customHeight="1">
       <c r="A29" t="s" s="8">
-        <v>1223</v>
+        <v>1230</v>
       </c>
       <c r="B29" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C29" s="16">
         <v>700</v>
@@ -47173,7 +47228,7 @@
         <v>5</v>
       </c>
       <c r="H29" t="s" s="17">
-        <v>1224</v>
+        <v>1231</v>
       </c>
       <c r="I29" s="10"/>
       <c r="J29" t="s" s="17">
@@ -47188,10 +47243,10 @@
     </row>
     <row r="30" ht="80.05" customHeight="1">
       <c r="A30" t="s" s="8">
-        <v>1225</v>
+        <v>1232</v>
       </c>
       <c r="B30" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C30" s="16">
         <v>1200</v>
@@ -47203,7 +47258,7 @@
         <v>4</v>
       </c>
       <c r="H30" t="s" s="17">
-        <v>1226</v>
+        <v>1233</v>
       </c>
       <c r="I30" s="10"/>
       <c r="J30" t="s" s="17">
@@ -47218,10 +47273,10 @@
     </row>
     <row r="31" ht="68.05" customHeight="1">
       <c r="A31" t="s" s="8">
-        <v>1227</v>
+        <v>1234</v>
       </c>
       <c r="B31" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C31" s="16">
         <v>1000</v>
@@ -47233,7 +47288,7 @@
         <v>5</v>
       </c>
       <c r="H31" t="s" s="17">
-        <v>1228</v>
+        <v>1235</v>
       </c>
       <c r="I31" s="10"/>
       <c r="J31" t="s" s="17">
@@ -47248,10 +47303,10 @@
     </row>
     <row r="32" ht="56.05" customHeight="1">
       <c r="A32" t="s" s="8">
-        <v>1229</v>
+        <v>1236</v>
       </c>
       <c r="B32" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C32" s="16">
         <v>1800</v>
@@ -47263,7 +47318,7 @@
         <v>5</v>
       </c>
       <c r="H32" t="s" s="17">
-        <v>1230</v>
+        <v>1237</v>
       </c>
       <c r="I32" s="10"/>
       <c r="J32" t="s" s="17">
@@ -47278,10 +47333,10 @@
     </row>
     <row r="33" ht="32.05" customHeight="1">
       <c r="A33" t="s" s="8">
-        <v>1231</v>
+        <v>1238</v>
       </c>
       <c r="B33" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C33" s="16">
         <v>1500</v>
@@ -47293,7 +47348,7 @@
         <v>4</v>
       </c>
       <c r="H33" t="s" s="17">
-        <v>1232</v>
+        <v>1239</v>
       </c>
       <c r="I33" s="10"/>
       <c r="J33" t="s" s="17">
@@ -47312,10 +47367,10 @@
     </row>
     <row r="34" ht="44.05" customHeight="1">
       <c r="A34" t="s" s="8">
-        <v>1233</v>
+        <v>1240</v>
       </c>
       <c r="B34" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C34" s="16">
         <v>1000</v>
@@ -47327,7 +47382,7 @@
         <v>3</v>
       </c>
       <c r="H34" t="s" s="17">
-        <v>1234</v>
+        <v>1241</v>
       </c>
       <c r="I34" s="10"/>
       <c r="J34" s="10"/>
@@ -47340,10 +47395,10 @@
     </row>
     <row r="35" ht="44.05" customHeight="1">
       <c r="A35" t="s" s="8">
-        <v>1235</v>
+        <v>1242</v>
       </c>
       <c r="B35" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C35" s="16">
         <v>600</v>
@@ -47355,7 +47410,7 @@
         <v>2</v>
       </c>
       <c r="H35" t="s" s="17">
-        <v>1236</v>
+        <v>1243</v>
       </c>
       <c r="I35" s="10"/>
       <c r="J35" s="10"/>
@@ -47368,10 +47423,10 @@
     </row>
     <row r="36" ht="56.05" customHeight="1">
       <c r="A36" t="s" s="8">
-        <v>1237</v>
+        <v>1244</v>
       </c>
       <c r="B36" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C36" s="16">
         <v>250</v>
@@ -47383,7 +47438,7 @@
         <v>3</v>
       </c>
       <c r="H36" t="s" s="17">
-        <v>1238</v>
+        <v>1245</v>
       </c>
       <c r="I36" s="10"/>
       <c r="J36" s="10"/>
@@ -47396,10 +47451,10 @@
     </row>
     <row r="37" ht="32.05" customHeight="1">
       <c r="A37" t="s" s="8">
-        <v>1239</v>
+        <v>1246</v>
       </c>
       <c r="B37" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C37" s="16">
         <v>300</v>
@@ -47411,7 +47466,7 @@
         <v>2</v>
       </c>
       <c r="H37" t="s" s="17">
-        <v>1240</v>
+        <v>1247</v>
       </c>
       <c r="I37" s="10"/>
       <c r="J37" s="10"/>
@@ -47424,10 +47479,10 @@
     </row>
     <row r="38" ht="44.05" customHeight="1">
       <c r="A38" t="s" s="8">
-        <v>1241</v>
+        <v>1248</v>
       </c>
       <c r="B38" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C38" s="16">
         <v>1000</v>
@@ -47439,7 +47494,7 @@
         <v>3</v>
       </c>
       <c r="H38" t="s" s="17">
-        <v>1242</v>
+        <v>1249</v>
       </c>
       <c r="I38" s="10"/>
       <c r="J38" s="10"/>
@@ -47452,10 +47507,10 @@
     </row>
     <row r="39" ht="32.05" customHeight="1">
       <c r="A39" t="s" s="8">
-        <v>1243</v>
+        <v>1250</v>
       </c>
       <c r="B39" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C39" s="16">
         <v>1200</v>
@@ -47467,7 +47522,7 @@
         <v>4</v>
       </c>
       <c r="H39" t="s" s="17">
-        <v>1244</v>
+        <v>1251</v>
       </c>
       <c r="I39" s="10"/>
       <c r="J39" s="10"/>
@@ -47480,10 +47535,10 @@
     </row>
     <row r="40" ht="20.05" customHeight="1">
       <c r="A40" t="s" s="8">
-        <v>1245</v>
+        <v>1252</v>
       </c>
       <c r="B40" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C40" s="16">
         <v>0</v>
@@ -47495,7 +47550,7 @@
         <v>1</v>
       </c>
       <c r="H40" t="s" s="17">
-        <v>1246</v>
+        <v>1253</v>
       </c>
       <c r="I40" s="10"/>
       <c r="J40" s="10"/>
@@ -47508,10 +47563,10 @@
     </row>
     <row r="41" ht="32.05" customHeight="1">
       <c r="A41" t="s" s="8">
-        <v>1247</v>
+        <v>1254</v>
       </c>
       <c r="B41" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C41" s="16">
         <v>0</v>
@@ -47523,7 +47578,7 @@
         <v>2</v>
       </c>
       <c r="H41" t="s" s="17">
-        <v>1248</v>
+        <v>1255</v>
       </c>
       <c r="I41" s="10"/>
       <c r="J41" s="10"/>
@@ -47536,10 +47591,10 @@
     </row>
     <row r="42" ht="32.05" customHeight="1">
       <c r="A42" t="s" s="8">
-        <v>1249</v>
+        <v>1256</v>
       </c>
       <c r="B42" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C42" s="16">
         <v>0</v>
@@ -47551,7 +47606,7 @@
         <v>1</v>
       </c>
       <c r="H42" t="s" s="17">
-        <v>1250</v>
+        <v>1257</v>
       </c>
       <c r="I42" s="10"/>
       <c r="J42" s="10"/>
@@ -47564,10 +47619,10 @@
     </row>
     <row r="43" ht="32.05" customHeight="1">
       <c r="A43" t="s" s="8">
-        <v>1251</v>
+        <v>1258</v>
       </c>
       <c r="B43" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C43" s="16">
         <v>0</v>
@@ -47579,7 +47634,7 @@
         <v>2</v>
       </c>
       <c r="H43" t="s" s="17">
-        <v>1252</v>
+        <v>1259</v>
       </c>
       <c r="I43" s="10"/>
       <c r="J43" s="10"/>
@@ -47592,10 +47647,10 @@
     </row>
     <row r="44" ht="20.05" customHeight="1">
       <c r="A44" t="s" s="8">
-        <v>1253</v>
+        <v>1260</v>
       </c>
       <c r="B44" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C44" s="16">
         <v>0</v>
@@ -47607,7 +47662,7 @@
         <v>1</v>
       </c>
       <c r="H44" t="s" s="17">
-        <v>1254</v>
+        <v>1261</v>
       </c>
       <c r="I44" s="10"/>
       <c r="J44" s="10"/>
@@ -47620,10 +47675,10 @@
     </row>
     <row r="45" ht="56.05" customHeight="1">
       <c r="A45" t="s" s="8">
-        <v>1255</v>
+        <v>1262</v>
       </c>
       <c r="B45" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C45" s="16">
         <v>0</v>
@@ -47635,7 +47690,7 @@
         <v>2</v>
       </c>
       <c r="H45" t="s" s="17">
-        <v>1256</v>
+        <v>1263</v>
       </c>
       <c r="I45" s="10"/>
       <c r="J45" s="10"/>
@@ -47648,10 +47703,10 @@
     </row>
     <row r="46" ht="44.05" customHeight="1">
       <c r="A46" t="s" s="8">
-        <v>1257</v>
+        <v>1264</v>
       </c>
       <c r="B46" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C46" s="16">
         <v>0</v>
@@ -47663,7 +47718,7 @@
         <v>1</v>
       </c>
       <c r="H46" t="s" s="17">
-        <v>1258</v>
+        <v>1265</v>
       </c>
       <c r="I46" s="10"/>
       <c r="J46" s="10"/>
@@ -47676,10 +47731,10 @@
     </row>
     <row r="47" ht="44.05" customHeight="1">
       <c r="A47" t="s" s="8">
-        <v>1259</v>
+        <v>1266</v>
       </c>
       <c r="B47" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C47" s="16">
         <v>0</v>
@@ -47691,7 +47746,7 @@
         <v>1</v>
       </c>
       <c r="H47" t="s" s="17">
-        <v>1260</v>
+        <v>1267</v>
       </c>
       <c r="I47" s="10"/>
       <c r="J47" s="10"/>
@@ -47704,10 +47759,10 @@
     </row>
     <row r="48" ht="56.05" customHeight="1">
       <c r="A48" t="s" s="8">
-        <v>1261</v>
+        <v>1268</v>
       </c>
       <c r="B48" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C48" s="16">
         <v>500</v>
@@ -47719,7 +47774,7 @@
         <v>1</v>
       </c>
       <c r="H48" t="s" s="17">
-        <v>1262</v>
+        <v>1269</v>
       </c>
       <c r="I48" s="10"/>
       <c r="J48" s="10"/>
@@ -47732,10 +47787,10 @@
     </row>
     <row r="49" ht="32.05" customHeight="1">
       <c r="A49" t="s" s="8">
-        <v>1263</v>
+        <v>1270</v>
       </c>
       <c r="B49" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C49" s="16">
         <v>0</v>
@@ -47747,7 +47802,7 @@
         <v>1</v>
       </c>
       <c r="H49" t="s" s="17">
-        <v>1264</v>
+        <v>1271</v>
       </c>
       <c r="I49" s="10"/>
       <c r="J49" s="10"/>
@@ -47760,10 +47815,10 @@
     </row>
     <row r="50" ht="32.05" customHeight="1">
       <c r="A50" t="s" s="8">
-        <v>1265</v>
+        <v>1272</v>
       </c>
       <c r="B50" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C50" s="16">
         <v>600</v>
@@ -47775,7 +47830,7 @@
         <v>1</v>
       </c>
       <c r="H50" t="s" s="17">
-        <v>1266</v>
+        <v>1273</v>
       </c>
       <c r="I50" s="10"/>
       <c r="J50" s="10"/>
@@ -47788,10 +47843,10 @@
     </row>
     <row r="51" ht="44.05" customHeight="1">
       <c r="A51" t="s" s="8">
-        <v>1267</v>
+        <v>1274</v>
       </c>
       <c r="B51" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C51" s="16">
         <v>0</v>
@@ -47803,7 +47858,7 @@
         <v>1</v>
       </c>
       <c r="H51" t="s" s="17">
-        <v>1268</v>
+        <v>1275</v>
       </c>
       <c r="I51" s="10"/>
       <c r="J51" s="10"/>
@@ -47816,10 +47871,10 @@
     </row>
     <row r="52" ht="68.05" customHeight="1">
       <c r="A52" t="s" s="8">
-        <v>1269</v>
+        <v>1276</v>
       </c>
       <c r="B52" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C52" s="16">
         <v>200</v>
@@ -47831,7 +47886,7 @@
         <v>1</v>
       </c>
       <c r="H52" t="s" s="17">
-        <v>1270</v>
+        <v>1277</v>
       </c>
       <c r="I52" s="10"/>
       <c r="J52" s="10"/>
@@ -47844,10 +47899,10 @@
     </row>
     <row r="53" ht="68.05" customHeight="1">
       <c r="A53" t="s" s="8">
-        <v>1271</v>
+        <v>1278</v>
       </c>
       <c r="B53" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C53" s="16">
         <v>200</v>
@@ -47859,7 +47914,7 @@
         <v>1</v>
       </c>
       <c r="H53" t="s" s="17">
-        <v>1272</v>
+        <v>1279</v>
       </c>
       <c r="I53" s="10"/>
       <c r="J53" s="10"/>
@@ -47872,10 +47927,10 @@
     </row>
     <row r="54" ht="80.05" customHeight="1">
       <c r="A54" t="s" s="8">
-        <v>1273</v>
+        <v>1280</v>
       </c>
       <c r="B54" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C54" s="16">
         <v>600</v>
@@ -47887,7 +47942,7 @@
         <v>1</v>
       </c>
       <c r="H54" t="s" s="17">
-        <v>1274</v>
+        <v>1281</v>
       </c>
       <c r="I54" s="10"/>
       <c r="J54" s="10"/>
@@ -47900,10 +47955,10 @@
     </row>
     <row r="55" ht="68.05" customHeight="1">
       <c r="A55" t="s" s="8">
-        <v>1275</v>
+        <v>1282</v>
       </c>
       <c r="B55" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C55" s="16">
         <v>500</v>
@@ -47915,7 +47970,7 @@
         <v>2</v>
       </c>
       <c r="H55" t="s" s="17">
-        <v>1276</v>
+        <v>1283</v>
       </c>
       <c r="I55" s="10"/>
       <c r="J55" s="10"/>
@@ -47928,10 +47983,10 @@
     </row>
     <row r="56" ht="44.05" customHeight="1">
       <c r="A56" t="s" s="8">
-        <v>1277</v>
+        <v>1284</v>
       </c>
       <c r="B56" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C56" s="16">
         <v>900</v>
@@ -47943,7 +47998,7 @@
         <v>2</v>
       </c>
       <c r="H56" t="s" s="17">
-        <v>1278</v>
+        <v>1285</v>
       </c>
       <c r="I56" s="10"/>
       <c r="J56" s="10"/>
@@ -47956,10 +48011,10 @@
     </row>
     <row r="57" ht="44.05" customHeight="1">
       <c r="A57" t="s" s="8">
-        <v>1279</v>
+        <v>1286</v>
       </c>
       <c r="B57" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C57" s="16">
         <v>0</v>
@@ -47971,7 +48026,7 @@
         <v>2</v>
       </c>
       <c r="H57" t="s" s="17">
-        <v>1280</v>
+        <v>1287</v>
       </c>
       <c r="I57" s="10"/>
       <c r="J57" s="10"/>
@@ -47984,10 +48039,10 @@
     </row>
     <row r="58" ht="56.05" customHeight="1">
       <c r="A58" t="s" s="8">
-        <v>1281</v>
+        <v>1288</v>
       </c>
       <c r="B58" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C58" s="16">
         <v>450</v>
@@ -47999,7 +48054,7 @@
         <v>2</v>
       </c>
       <c r="H58" t="s" s="17">
-        <v>1282</v>
+        <v>1289</v>
       </c>
       <c r="I58" s="10"/>
       <c r="J58" s="10"/>
@@ -48012,10 +48067,10 @@
     </row>
     <row r="59" ht="68.05" customHeight="1">
       <c r="A59" t="s" s="8">
-        <v>1283</v>
+        <v>1290</v>
       </c>
       <c r="B59" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C59" s="16">
         <v>450</v>
@@ -48027,7 +48082,7 @@
         <v>2</v>
       </c>
       <c r="H59" t="s" s="17">
-        <v>1284</v>
+        <v>1291</v>
       </c>
       <c r="I59" s="10"/>
       <c r="J59" s="10"/>
@@ -48040,10 +48095,10 @@
     </row>
     <row r="60" ht="44.05" customHeight="1">
       <c r="A60" t="s" s="8">
-        <v>1285</v>
+        <v>1292</v>
       </c>
       <c r="B60" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C60" s="16">
         <v>200</v>
@@ -48055,7 +48110,7 @@
         <v>4</v>
       </c>
       <c r="H60" t="s" s="17">
-        <v>1286</v>
+        <v>1293</v>
       </c>
       <c r="I60" s="10"/>
       <c r="J60" s="10"/>
@@ -48068,10 +48123,10 @@
     </row>
     <row r="61" ht="32.05" customHeight="1">
       <c r="A61" t="s" s="8">
-        <v>1287</v>
+        <v>1294</v>
       </c>
       <c r="B61" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C61" s="16">
         <v>1200</v>
@@ -48083,7 +48138,7 @@
         <v>5</v>
       </c>
       <c r="H61" t="s" s="17">
-        <v>1288</v>
+        <v>1295</v>
       </c>
       <c r="I61" s="10"/>
       <c r="J61" s="10"/>
@@ -48096,10 +48151,10 @@
     </row>
     <row r="62" ht="44.05" customHeight="1">
       <c r="A62" t="s" s="8">
-        <v>1289</v>
+        <v>1296</v>
       </c>
       <c r="B62" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C62" s="16">
         <v>0</v>
@@ -48111,7 +48166,7 @@
         <v>2</v>
       </c>
       <c r="H62" t="s" s="17">
-        <v>1290</v>
+        <v>1297</v>
       </c>
       <c r="I62" s="10"/>
       <c r="J62" s="10"/>
@@ -48124,10 +48179,10 @@
     </row>
     <row r="63" ht="32.05" customHeight="1">
       <c r="A63" t="s" s="8">
-        <v>1291</v>
+        <v>1298</v>
       </c>
       <c r="B63" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C63" s="16">
         <v>0</v>
@@ -48139,7 +48194,7 @@
         <v>4</v>
       </c>
       <c r="H63" t="s" s="17">
-        <v>1292</v>
+        <v>1299</v>
       </c>
       <c r="I63" s="10"/>
       <c r="J63" s="10"/>
@@ -48152,10 +48207,10 @@
     </row>
     <row r="64" ht="32.05" customHeight="1">
       <c r="A64" t="s" s="8">
-        <v>1293</v>
+        <v>1300</v>
       </c>
       <c r="B64" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C64" s="16">
         <v>0</v>
@@ -48167,7 +48222,7 @@
         <v>4</v>
       </c>
       <c r="H64" t="s" s="17">
-        <v>1294</v>
+        <v>1301</v>
       </c>
       <c r="I64" s="10"/>
       <c r="J64" s="10"/>
@@ -48180,10 +48235,10 @@
     </row>
     <row r="65" ht="80.05" customHeight="1">
       <c r="A65" t="s" s="8">
-        <v>1295</v>
+        <v>1302</v>
       </c>
       <c r="B65" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C65" s="16">
         <v>800</v>
@@ -48195,7 +48250,7 @@
         <v>3</v>
       </c>
       <c r="H65" t="s" s="17">
-        <v>1296</v>
+        <v>1303</v>
       </c>
       <c r="I65" s="10"/>
       <c r="J65" s="10"/>
@@ -48208,10 +48263,10 @@
     </row>
     <row r="66" ht="80.05" customHeight="1">
       <c r="A66" t="s" s="8">
-        <v>1297</v>
+        <v>1304</v>
       </c>
       <c r="B66" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C66" s="16">
         <v>800</v>
@@ -48223,7 +48278,7 @@
         <v>2</v>
       </c>
       <c r="H66" t="s" s="17">
-        <v>1298</v>
+        <v>1305</v>
       </c>
       <c r="I66" s="10"/>
       <c r="J66" s="10"/>
@@ -48236,10 +48291,10 @@
     </row>
     <row r="67" ht="68.05" customHeight="1">
       <c r="A67" t="s" s="8">
-        <v>1299</v>
+        <v>1306</v>
       </c>
       <c r="B67" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C67" s="16">
         <v>1000</v>
@@ -48251,7 +48306,7 @@
         <v>5</v>
       </c>
       <c r="H67" t="s" s="17">
-        <v>1300</v>
+        <v>1307</v>
       </c>
       <c r="I67" s="10"/>
       <c r="J67" s="10"/>
@@ -48264,10 +48319,10 @@
     </row>
     <row r="68" ht="56.05" customHeight="1">
       <c r="A68" t="s" s="8">
-        <v>1301</v>
+        <v>1308</v>
       </c>
       <c r="B68" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C68" s="16">
         <v>1500</v>
@@ -48279,7 +48334,7 @@
         <v>3</v>
       </c>
       <c r="H68" t="s" s="17">
-        <v>1302</v>
+        <v>1309</v>
       </c>
       <c r="I68" s="10"/>
       <c r="J68" s="10"/>
@@ -48292,10 +48347,10 @@
     </row>
     <row r="69" ht="44.05" customHeight="1">
       <c r="A69" t="s" s="8">
-        <v>1303</v>
+        <v>1310</v>
       </c>
       <c r="B69" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C69" s="16">
         <v>1200</v>
@@ -48307,7 +48362,7 @@
         <v>2</v>
       </c>
       <c r="H69" t="s" s="17">
-        <v>1304</v>
+        <v>1311</v>
       </c>
       <c r="I69" s="10"/>
       <c r="J69" s="10"/>
@@ -48320,10 +48375,10 @@
     </row>
     <row r="70" ht="56.05" customHeight="1">
       <c r="A70" t="s" s="8">
-        <v>1305</v>
+        <v>1312</v>
       </c>
       <c r="B70" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C70" s="16">
         <v>300</v>
@@ -48335,7 +48390,7 @@
         <v>1</v>
       </c>
       <c r="H70" t="s" s="17">
-        <v>1306</v>
+        <v>1313</v>
       </c>
       <c r="I70" s="10"/>
       <c r="J70" s="10"/>
@@ -48348,10 +48403,10 @@
     </row>
     <row r="71" ht="68.05" customHeight="1">
       <c r="A71" t="s" s="8">
-        <v>1307</v>
+        <v>1314</v>
       </c>
       <c r="B71" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C71" s="16">
         <v>300</v>
@@ -48363,7 +48418,7 @@
         <v>1</v>
       </c>
       <c r="H71" t="s" s="17">
-        <v>1308</v>
+        <v>1315</v>
       </c>
       <c r="I71" s="10"/>
       <c r="J71" s="10"/>
@@ -48376,10 +48431,10 @@
     </row>
     <row r="72" ht="68.05" customHeight="1">
       <c r="A72" t="s" s="8">
-        <v>1309</v>
+        <v>1316</v>
       </c>
       <c r="B72" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C72" s="16">
         <v>500</v>
@@ -48391,7 +48446,7 @@
         <v>2</v>
       </c>
       <c r="H72" t="s" s="17">
-        <v>1310</v>
+        <v>1317</v>
       </c>
       <c r="I72" s="10"/>
       <c r="J72" s="10"/>
@@ -48404,10 +48459,10 @@
     </row>
     <row r="73" ht="44.05" customHeight="1">
       <c r="A73" t="s" s="8">
-        <v>1311</v>
+        <v>1318</v>
       </c>
       <c r="B73" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C73" s="16">
         <v>2000</v>
@@ -48419,7 +48474,7 @@
         <v>4</v>
       </c>
       <c r="H73" t="s" s="17">
-        <v>1312</v>
+        <v>1319</v>
       </c>
       <c r="I73" s="10"/>
       <c r="J73" s="10"/>
@@ -48432,10 +48487,10 @@
     </row>
     <row r="74" ht="44.05" customHeight="1">
       <c r="A74" t="s" s="8">
-        <v>1313</v>
+        <v>1320</v>
       </c>
       <c r="B74" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C74" s="16">
         <v>2000</v>
@@ -48447,7 +48502,7 @@
         <v>5</v>
       </c>
       <c r="H74" t="s" s="17">
-        <v>1314</v>
+        <v>1321</v>
       </c>
       <c r="I74" s="10"/>
       <c r="J74" s="10"/>
@@ -48460,10 +48515,10 @@
     </row>
     <row r="75" ht="44.05" customHeight="1">
       <c r="A75" t="s" s="8">
-        <v>1315</v>
+        <v>1322</v>
       </c>
       <c r="B75" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C75" s="16">
         <v>2000</v>
@@ -48475,7 +48530,7 @@
         <v>5</v>
       </c>
       <c r="H75" t="s" s="17">
-        <v>1316</v>
+        <v>1323</v>
       </c>
       <c r="I75" s="10"/>
       <c r="J75" s="10"/>
@@ -48488,10 +48543,10 @@
     </row>
     <row r="76" ht="44.05" customHeight="1">
       <c r="A76" t="s" s="8">
-        <v>1317</v>
+        <v>1324</v>
       </c>
       <c r="B76" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C76" s="16">
         <v>2000</v>
@@ -48503,7 +48558,7 @@
         <v>5</v>
       </c>
       <c r="H76" t="s" s="17">
-        <v>1318</v>
+        <v>1325</v>
       </c>
       <c r="I76" s="10"/>
       <c r="J76" s="10"/>
@@ -48516,10 +48571,10 @@
     </row>
     <row r="77" ht="44.05" customHeight="1">
       <c r="A77" t="s" s="8">
-        <v>1319</v>
+        <v>1326</v>
       </c>
       <c r="B77" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C77" s="16">
         <v>2000</v>
@@ -48531,7 +48586,7 @@
         <v>5</v>
       </c>
       <c r="H77" t="s" s="17">
-        <v>1320</v>
+        <v>1327</v>
       </c>
       <c r="I77" s="10"/>
       <c r="J77" s="10"/>
@@ -48544,10 +48599,10 @@
     </row>
     <row r="78" ht="44.05" customHeight="1">
       <c r="A78" t="s" s="8">
-        <v>1321</v>
+        <v>1328</v>
       </c>
       <c r="B78" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C78" s="16">
         <v>2000</v>
@@ -48559,7 +48614,7 @@
         <v>5</v>
       </c>
       <c r="H78" t="s" s="17">
-        <v>1322</v>
+        <v>1329</v>
       </c>
       <c r="I78" s="10"/>
       <c r="J78" s="10"/>
@@ -48572,10 +48627,10 @@
     </row>
     <row r="79" ht="44.05" customHeight="1">
       <c r="A79" t="s" s="8">
-        <v>1323</v>
+        <v>1330</v>
       </c>
       <c r="B79" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C79" s="16">
         <v>2000</v>
@@ -48587,7 +48642,7 @@
         <v>5</v>
       </c>
       <c r="H79" t="s" s="17">
-        <v>1324</v>
+        <v>1331</v>
       </c>
       <c r="I79" s="10"/>
       <c r="J79" s="10"/>
@@ -48600,10 +48655,10 @@
     </row>
     <row r="80" ht="20.05" customHeight="1">
       <c r="A80" t="s" s="8">
-        <v>1325</v>
+        <v>1332</v>
       </c>
       <c r="B80" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C80" s="16">
         <v>1200</v>
@@ -48615,7 +48670,7 @@
         <v>4</v>
       </c>
       <c r="H80" t="s" s="17">
-        <v>1326</v>
+        <v>1333</v>
       </c>
       <c r="I80" s="10"/>
       <c r="J80" s="10"/>
@@ -48628,10 +48683,10 @@
     </row>
     <row r="81" ht="56.05" customHeight="1">
       <c r="A81" t="s" s="8">
-        <v>1327</v>
+        <v>1334</v>
       </c>
       <c r="B81" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C81" s="16">
         <v>2000</v>
@@ -48643,7 +48698,7 @@
         <v>3</v>
       </c>
       <c r="H81" t="s" s="17">
-        <v>1328</v>
+        <v>1335</v>
       </c>
       <c r="I81" s="10"/>
       <c r="J81" s="10"/>
@@ -48656,10 +48711,10 @@
     </row>
     <row r="82" ht="44.05" customHeight="1">
       <c r="A82" t="s" s="8">
-        <v>1329</v>
+        <v>1336</v>
       </c>
       <c r="B82" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C82" s="16">
         <v>1000</v>
@@ -48671,7 +48726,7 @@
         <v>3</v>
       </c>
       <c r="H82" t="s" s="17">
-        <v>1330</v>
+        <v>1337</v>
       </c>
       <c r="I82" s="10"/>
       <c r="J82" s="10"/>
@@ -48684,10 +48739,10 @@
     </row>
     <row r="83" ht="32.05" customHeight="1">
       <c r="A83" t="s" s="8">
-        <v>1331</v>
+        <v>1338</v>
       </c>
       <c r="B83" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C83" s="16">
         <v>500</v>
@@ -48699,7 +48754,7 @@
         <v>2</v>
       </c>
       <c r="H83" t="s" s="17">
-        <v>1332</v>
+        <v>1339</v>
       </c>
       <c r="I83" s="10"/>
       <c r="J83" s="10"/>
@@ -48712,10 +48767,10 @@
     </row>
     <row r="84" ht="32.05" customHeight="1">
       <c r="A84" t="s" s="8">
-        <v>1333</v>
+        <v>1340</v>
       </c>
       <c r="B84" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C84" s="16">
         <v>250</v>
@@ -48727,7 +48782,7 @@
         <v>1</v>
       </c>
       <c r="H84" t="s" s="17">
-        <v>1334</v>
+        <v>1341</v>
       </c>
       <c r="I84" s="10"/>
       <c r="J84" s="10"/>
@@ -48740,10 +48795,10 @@
     </row>
     <row r="85" ht="80.05" customHeight="1">
       <c r="A85" t="s" s="8">
-        <v>1335</v>
+        <v>1342</v>
       </c>
       <c r="B85" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C85" s="16">
         <v>1500</v>
@@ -48755,7 +48810,7 @@
         <v>4</v>
       </c>
       <c r="H85" t="s" s="17">
-        <v>1336</v>
+        <v>1343</v>
       </c>
       <c r="I85" s="10"/>
       <c r="J85" s="10"/>
@@ -48768,10 +48823,10 @@
     </row>
     <row r="86" ht="32.05" customHeight="1">
       <c r="A86" t="s" s="8">
-        <v>1337</v>
+        <v>1344</v>
       </c>
       <c r="B86" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C86" s="16">
         <v>1000</v>
@@ -48783,7 +48838,7 @@
         <v>3</v>
       </c>
       <c r="H86" t="s" s="17">
-        <v>1338</v>
+        <v>1345</v>
       </c>
       <c r="I86" s="10"/>
       <c r="J86" s="10"/>
@@ -48796,10 +48851,10 @@
     </row>
     <row r="87" ht="44.05" customHeight="1">
       <c r="A87" t="s" s="8">
-        <v>1339</v>
+        <v>1346</v>
       </c>
       <c r="B87" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C87" s="16">
         <v>800</v>
@@ -48811,7 +48866,7 @@
         <v>2</v>
       </c>
       <c r="H87" t="s" s="17">
-        <v>1340</v>
+        <v>1347</v>
       </c>
       <c r="I87" s="10"/>
       <c r="J87" s="10"/>
@@ -48824,10 +48879,10 @@
     </row>
     <row r="88" ht="32.05" customHeight="1">
       <c r="A88" t="s" s="8">
-        <v>1341</v>
+        <v>1348</v>
       </c>
       <c r="B88" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C88" s="16">
         <v>200</v>
@@ -48839,7 +48894,7 @@
         <v>2</v>
       </c>
       <c r="H88" t="s" s="17">
-        <v>1342</v>
+        <v>1349</v>
       </c>
       <c r="I88" s="10"/>
       <c r="J88" s="10"/>
@@ -48852,10 +48907,10 @@
     </row>
     <row r="89" ht="32.05" customHeight="1">
       <c r="A89" t="s" s="8">
-        <v>1343</v>
+        <v>1350</v>
       </c>
       <c r="B89" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C89" s="16">
         <v>1500</v>
@@ -48867,7 +48922,7 @@
         <v>3</v>
       </c>
       <c r="H89" t="s" s="17">
-        <v>1344</v>
+        <v>1351</v>
       </c>
       <c r="I89" s="10"/>
       <c r="J89" s="10"/>
@@ -48880,10 +48935,10 @@
     </row>
     <row r="90" ht="32.05" customHeight="1">
       <c r="A90" t="s" s="8">
-        <v>1345</v>
+        <v>1352</v>
       </c>
       <c r="B90" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C90" s="16">
         <v>500</v>
@@ -48895,7 +48950,7 @@
         <v>5</v>
       </c>
       <c r="H90" t="s" s="17">
-        <v>1346</v>
+        <v>1353</v>
       </c>
       <c r="I90" s="10"/>
       <c r="J90" s="10"/>
@@ -48908,10 +48963,10 @@
     </row>
     <row r="91" ht="80.05" customHeight="1">
       <c r="A91" t="s" s="8">
-        <v>1347</v>
+        <v>1354</v>
       </c>
       <c r="B91" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C91" s="16">
         <v>1000</v>
@@ -48923,11 +48978,11 @@
         <v>2</v>
       </c>
       <c r="H91" t="s" s="17">
-        <v>1348</v>
+        <v>1355</v>
       </c>
       <c r="I91" s="10"/>
       <c r="J91" t="s" s="17">
-        <v>1349</v>
+        <v>1356</v>
       </c>
       <c r="K91" s="10"/>
       <c r="L91" s="10"/>
@@ -48938,10 +48993,10 @@
     </row>
     <row r="92" ht="56.05" customHeight="1">
       <c r="A92" t="s" s="8">
-        <v>1350</v>
+        <v>1357</v>
       </c>
       <c r="B92" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C92" s="16">
         <v>1500</v>
@@ -48953,7 +49008,7 @@
         <v>4</v>
       </c>
       <c r="H92" t="s" s="17">
-        <v>1351</v>
+        <v>1358</v>
       </c>
       <c r="I92" s="10"/>
       <c r="J92" s="10"/>
@@ -48966,10 +49021,10 @@
     </row>
     <row r="93" ht="44.05" customHeight="1">
       <c r="A93" t="s" s="8">
-        <v>1352</v>
+        <v>1359</v>
       </c>
       <c r="B93" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C93" s="16">
         <v>300</v>
@@ -48981,7 +49036,7 @@
         <v>1</v>
       </c>
       <c r="H93" t="s" s="17">
-        <v>1353</v>
+        <v>1360</v>
       </c>
       <c r="I93" s="10"/>
       <c r="J93" s="10"/>
@@ -48994,10 +49049,10 @@
     </row>
     <row r="94" ht="68.05" customHeight="1">
       <c r="A94" t="s" s="8">
-        <v>1354</v>
+        <v>1361</v>
       </c>
       <c r="B94" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C94" s="16">
         <v>200</v>
@@ -49009,7 +49064,7 @@
         <v>1</v>
       </c>
       <c r="H94" t="s" s="17">
-        <v>1355</v>
+        <v>1362</v>
       </c>
       <c r="I94" s="10"/>
       <c r="J94" s="10"/>
@@ -49022,10 +49077,10 @@
     </row>
     <row r="95" ht="68.05" customHeight="1">
       <c r="A95" t="s" s="8">
-        <v>1356</v>
+        <v>1363</v>
       </c>
       <c r="B95" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C95" s="16">
         <v>0</v>
@@ -49037,7 +49092,7 @@
         <v>1</v>
       </c>
       <c r="H95" t="s" s="17">
-        <v>1357</v>
+        <v>1364</v>
       </c>
       <c r="I95" s="10"/>
       <c r="J95" s="10"/>
@@ -49050,10 +49105,10 @@
     </row>
     <row r="96" ht="44.05" customHeight="1">
       <c r="A96" t="s" s="8">
-        <v>1358</v>
+        <v>1365</v>
       </c>
       <c r="B96" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C96" s="16">
         <v>0</v>
@@ -49065,7 +49120,7 @@
         <v>1</v>
       </c>
       <c r="H96" t="s" s="17">
-        <v>1359</v>
+        <v>1366</v>
       </c>
       <c r="I96" s="10"/>
       <c r="J96" s="10"/>
@@ -49078,10 +49133,10 @@
     </row>
     <row r="97" ht="44.05" customHeight="1">
       <c r="A97" t="s" s="8">
-        <v>1360</v>
+        <v>1367</v>
       </c>
       <c r="B97" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C97" s="16">
         <v>1000</v>
@@ -49093,7 +49148,7 @@
         <v>1</v>
       </c>
       <c r="H97" t="s" s="17">
-        <v>1361</v>
+        <v>1368</v>
       </c>
       <c r="I97" s="10"/>
       <c r="J97" s="10"/>
@@ -49106,10 +49161,10 @@
     </row>
     <row r="98" ht="32.05" customHeight="1">
       <c r="A98" t="s" s="8">
-        <v>1362</v>
+        <v>1369</v>
       </c>
       <c r="B98" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C98" s="16">
         <v>0</v>
@@ -49121,7 +49176,7 @@
         <v>1</v>
       </c>
       <c r="H98" t="s" s="17">
-        <v>1363</v>
+        <v>1370</v>
       </c>
       <c r="I98" s="10"/>
       <c r="J98" s="10"/>
@@ -49134,10 +49189,10 @@
     </row>
     <row r="99" ht="44.05" customHeight="1">
       <c r="A99" t="s" s="8">
-        <v>1364</v>
+        <v>1371</v>
       </c>
       <c r="B99" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C99" s="16">
         <v>0</v>
@@ -49149,7 +49204,7 @@
         <v>1</v>
       </c>
       <c r="H99" t="s" s="17">
-        <v>1365</v>
+        <v>1372</v>
       </c>
       <c r="I99" s="10"/>
       <c r="J99" s="10"/>
@@ -49162,10 +49217,10 @@
     </row>
     <row r="100" ht="44.05" customHeight="1">
       <c r="A100" t="s" s="8">
-        <v>1366</v>
+        <v>1373</v>
       </c>
       <c r="B100" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C100" s="16">
         <v>500</v>
@@ -49177,7 +49232,7 @@
         <v>2</v>
       </c>
       <c r="H100" t="s" s="17">
-        <v>1367</v>
+        <v>1374</v>
       </c>
       <c r="I100" s="10"/>
       <c r="J100" s="10"/>
@@ -49190,10 +49245,10 @@
     </row>
     <row r="101" ht="44.05" customHeight="1">
       <c r="A101" t="s" s="8">
-        <v>1368</v>
+        <v>1375</v>
       </c>
       <c r="B101" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C101" s="16">
         <v>0</v>
@@ -49205,7 +49260,7 @@
         <v>2</v>
       </c>
       <c r="H101" t="s" s="17">
-        <v>1369</v>
+        <v>1376</v>
       </c>
       <c r="I101" s="10"/>
       <c r="J101" s="10"/>
@@ -49218,10 +49273,10 @@
     </row>
     <row r="102" ht="44.05" customHeight="1">
       <c r="A102" t="s" s="8">
-        <v>1370</v>
+        <v>1377</v>
       </c>
       <c r="B102" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C102" s="16">
         <v>600</v>
@@ -49233,7 +49288,7 @@
         <v>2</v>
       </c>
       <c r="H102" t="s" s="17">
-        <v>1371</v>
+        <v>1378</v>
       </c>
       <c r="I102" s="10"/>
       <c r="J102" s="10"/>
@@ -49246,10 +49301,10 @@
     </row>
     <row r="103" ht="92.05" customHeight="1">
       <c r="A103" t="s" s="8">
-        <v>1372</v>
+        <v>1379</v>
       </c>
       <c r="B103" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C103" s="16">
         <v>500</v>
@@ -49261,7 +49316,7 @@
         <v>2</v>
       </c>
       <c r="H103" t="s" s="17">
-        <v>1373</v>
+        <v>1380</v>
       </c>
       <c r="I103" s="10"/>
       <c r="J103" s="10"/>
@@ -49274,10 +49329,10 @@
     </row>
     <row r="104" ht="56.05" customHeight="1">
       <c r="A104" t="s" s="8">
-        <v>1374</v>
+        <v>1381</v>
       </c>
       <c r="B104" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C104" s="16">
         <v>2000</v>
@@ -49289,7 +49344,7 @@
         <v>4</v>
       </c>
       <c r="H104" t="s" s="17">
-        <v>1375</v>
+        <v>1382</v>
       </c>
       <c r="I104" s="10"/>
       <c r="J104" t="s" s="17">
@@ -49304,10 +49359,10 @@
     </row>
     <row r="105" ht="32.05" customHeight="1">
       <c r="A105" t="s" s="8">
-        <v>1376</v>
+        <v>1383</v>
       </c>
       <c r="B105" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C105" s="16">
         <v>1500</v>
@@ -49319,7 +49374,7 @@
         <v>4</v>
       </c>
       <c r="H105" t="s" s="17">
-        <v>1377</v>
+        <v>1384</v>
       </c>
       <c r="I105" s="10"/>
       <c r="J105" s="10"/>
@@ -49332,10 +49387,10 @@
     </row>
     <row r="106" ht="32.05" customHeight="1">
       <c r="A106" t="s" s="8">
-        <v>1378</v>
+        <v>1385</v>
       </c>
       <c r="B106" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C106" s="16">
         <v>0</v>
@@ -49347,7 +49402,7 @@
         <v>1</v>
       </c>
       <c r="H106" t="s" s="17">
-        <v>1379</v>
+        <v>1386</v>
       </c>
       <c r="I106" s="10"/>
       <c r="J106" s="10"/>
@@ -49360,10 +49415,10 @@
     </row>
     <row r="107" ht="68.05" customHeight="1">
       <c r="A107" t="s" s="8">
-        <v>1380</v>
+        <v>1387</v>
       </c>
       <c r="B107" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C107" s="16">
         <v>2000</v>
@@ -49375,7 +49430,7 @@
         <v>3</v>
       </c>
       <c r="H107" t="s" s="17">
-        <v>1381</v>
+        <v>1388</v>
       </c>
       <c r="I107" s="10"/>
       <c r="J107" s="10"/>
@@ -49388,10 +49443,10 @@
     </row>
     <row r="108" ht="44.05" customHeight="1">
       <c r="A108" t="s" s="8">
-        <v>1382</v>
+        <v>1389</v>
       </c>
       <c r="B108" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C108" s="16">
         <v>300</v>
@@ -49401,7 +49456,7 @@
       <c r="F108" s="10"/>
       <c r="G108" s="10"/>
       <c r="H108" t="s" s="17">
-        <v>1383</v>
+        <v>1390</v>
       </c>
       <c r="I108" s="10"/>
       <c r="J108" s="10"/>
@@ -49414,10 +49469,10 @@
     </row>
     <row r="109" ht="56.05" customHeight="1">
       <c r="A109" t="s" s="8">
-        <v>1384</v>
+        <v>1391</v>
       </c>
       <c r="B109" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C109" s="16">
         <v>800</v>
@@ -49427,7 +49482,7 @@
       <c r="F109" s="10"/>
       <c r="G109" s="10"/>
       <c r="H109" t="s" s="17">
-        <v>1385</v>
+        <v>1392</v>
       </c>
       <c r="I109" s="10"/>
       <c r="J109" s="10"/>
@@ -49440,10 +49495,10 @@
     </row>
     <row r="110" ht="56.05" customHeight="1">
       <c r="A110" t="s" s="8">
-        <v>1386</v>
+        <v>1393</v>
       </c>
       <c r="B110" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C110" s="16">
         <v>600</v>
@@ -49453,7 +49508,7 @@
       <c r="F110" s="10"/>
       <c r="G110" s="10"/>
       <c r="H110" t="s" s="17">
-        <v>1387</v>
+        <v>1394</v>
       </c>
       <c r="I110" s="10"/>
       <c r="J110" s="10"/>
@@ -49466,10 +49521,10 @@
     </row>
     <row r="111" ht="56.05" customHeight="1">
       <c r="A111" t="s" s="8">
-        <v>1388</v>
+        <v>1395</v>
       </c>
       <c r="B111" t="s" s="9">
-        <v>1171</v>
+        <v>1178</v>
       </c>
       <c r="C111" s="16">
         <v>300</v>
@@ -49479,7 +49534,7 @@
       <c r="F111" s="10"/>
       <c r="G111" s="10"/>
       <c r="H111" t="s" s="17">
-        <v>1389</v>
+        <v>1396</v>
       </c>
       <c r="I111" s="10"/>
       <c r="J111" s="10"/>
@@ -57539,21 +57594,21 @@
         <v>22</v>
       </c>
       <c r="B2" t="s" s="22">
-        <v>1390</v>
+        <v>1397</v>
       </c>
       <c r="C2" t="s" s="22">
-        <v>1391</v>
+        <v>1398</v>
       </c>
       <c r="D2" t="s" s="22">
-        <v>1392</v>
+        <v>1399</v>
       </c>
       <c r="E2" t="s" s="22">
-        <v>1393</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="3" ht="16.55" customHeight="1">
       <c r="A3" t="s" s="23">
-        <v>1394</v>
+        <v>1401</v>
       </c>
       <c r="B3" s="24">
         <v>52</v>
@@ -57562,7 +57617,7 @@
         <v>0.347</v>
       </c>
       <c r="D3" t="s" s="26">
-        <v>1395</v>
+        <v>1402</v>
       </c>
       <c r="E3" s="27">
         <f>_xlfn.COUNTIFS('Unit'!$L$3:$L$568,"Yes",'Unit'!$G$3:$G$568,1)+_xlfn.COUNTIFS('Trap'!$L$3:$L$545,"Yes",'Trap'!$G$3:$G$545,1)+_xlfn.COUNTIFS('Tech'!$L$3:$L$556,"Yes",'Tech'!$G$3:$G$556,1)</f>
@@ -57571,7 +57626,7 @@
     </row>
     <row r="4" ht="16.35" customHeight="1">
       <c r="A4" t="s" s="28">
-        <v>1396</v>
+        <v>1403</v>
       </c>
       <c r="B4" s="29">
         <v>48</v>
@@ -57580,7 +57635,7 @@
         <v>0.337</v>
       </c>
       <c r="D4" t="s" s="31">
-        <v>1397</v>
+        <v>1404</v>
       </c>
       <c r="E4" s="32">
         <f>_xlfn.COUNTIFS('Unit'!$L$3:$L$568,"Yes",'Unit'!$G$3:$G$568,2)+_xlfn.COUNTIFS('Trap'!$L$3:$L$545,"Yes",'Trap'!$G$3:$G$545,2)+_xlfn.COUNTIFS('Tech'!$L$3:$L$556,"Yes",'Tech'!$G$3:$G$556,2)</f>
@@ -57589,7 +57644,7 @@
     </row>
     <row r="5" ht="16.35" customHeight="1">
       <c r="A5" t="s" s="28">
-        <v>1398</v>
+        <v>1405</v>
       </c>
       <c r="B5" s="29">
         <v>27</v>
@@ -57598,7 +57653,7 @@
         <v>0.167</v>
       </c>
       <c r="D5" t="s" s="31">
-        <v>1397</v>
+        <v>1404</v>
       </c>
       <c r="E5" s="32">
         <f>_xlfn.COUNTIFS('Unit'!$L$3:$L$568,"Yes",'Unit'!$G$3:$G$568,3)+_xlfn.COUNTIFS('Trap'!$L$3:$L$545,"Yes",'Trap'!$G$3:$G$545,3)+_xlfn.COUNTIFS('Tech'!$L$3:$L$556,"Yes",'Tech'!$G$3:$G$556,3)</f>
@@ -57607,7 +57662,7 @@
     </row>
     <row r="6" ht="30.35" customHeight="1">
       <c r="A6" t="s" s="28">
-        <v>1399</v>
+        <v>1406</v>
       </c>
       <c r="B6" s="29">
         <v>16</v>
@@ -57616,7 +57671,7 @@
         <v>0.1</v>
       </c>
       <c r="D6" t="s" s="31">
-        <v>1400</v>
+        <v>1407</v>
       </c>
       <c r="E6" s="32">
         <f>_xlfn.COUNTIFS('Unit'!$L$3:$L$568,"Yes",'Unit'!$G$3:$G$568,4)+_xlfn.COUNTIFS('Trap'!$L$3:$L$545,"Yes",'Trap'!$G$3:$G$545,4)+_xlfn.COUNTIFS('Tech'!$L$3:$L$556,"Yes",'Tech'!$G$3:$G$556,4)</f>
@@ -57625,7 +57680,7 @@
     </row>
     <row r="7" ht="16.35" customHeight="1">
       <c r="A7" t="s" s="33">
-        <v>1401</v>
+        <v>1408</v>
       </c>
       <c r="B7" s="34">
         <v>9</v>
@@ -57634,7 +57689,7 @@
         <v>0.053</v>
       </c>
       <c r="D7" t="s" s="31">
-        <v>1402</v>
+        <v>1409</v>
       </c>
       <c r="E7" s="32">
         <f>_xlfn.COUNTIFS('Unit'!$L$3:$L$568,"Yes",'Unit'!$G$3:$G$568,5)+_xlfn.COUNTIFS('Trap'!$L$3:$L$545,"Yes",'Trap'!$G$3:$G$545,5)+_xlfn.COUNTIFS('Tech'!$L$3:$L$556,"Yes",'Tech'!$G$3:$G$556,5)</f>
@@ -57667,17 +57722,17 @@
         <v>22</v>
       </c>
       <c r="B11" t="s" s="41">
-        <v>1390</v>
+        <v>1397</v>
       </c>
       <c r="C11" s="42"/>
       <c r="D11" s="42"/>
       <c r="E11" t="s" s="43">
-        <v>1393</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="12" ht="16.35" customHeight="1">
       <c r="A12" t="s" s="28">
-        <v>1403</v>
+        <v>1410</v>
       </c>
       <c r="B12" s="29">
         <v>60</v>
@@ -57691,7 +57746,7 @@
     </row>
     <row r="13" ht="16.35" customHeight="1">
       <c r="A13" t="s" s="28">
-        <v>1404</v>
+        <v>1411</v>
       </c>
       <c r="B13" s="29">
         <v>60</v>
@@ -57705,7 +57760,7 @@
     </row>
     <row r="14" ht="16.35" customHeight="1">
       <c r="A14" t="s" s="28">
-        <v>1405</v>
+        <v>1412</v>
       </c>
       <c r="B14" s="29">
         <v>60</v>
@@ -57753,10 +57808,10 @@
     <row r="2" ht="20.25" customHeight="1">
       <c r="A2" s="4"/>
       <c r="B2" t="s" s="3">
-        <v>1406</v>
+        <v>1413</v>
       </c>
       <c r="C2" t="s" s="3">
-        <v>1407</v>
+        <v>1414</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -57766,10 +57821,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s" s="6">
-        <v>1408</v>
+        <v>1415</v>
       </c>
       <c r="C3" t="s" s="15">
-        <v>1409</v>
+        <v>1416</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -57779,10 +57834,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s" s="9">
-        <v>1410</v>
+        <v>1417</v>
       </c>
       <c r="C4" t="s" s="17">
-        <v>1411</v>
+        <v>1418</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -57792,10 +57847,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s" s="9">
-        <v>1412</v>
+        <v>1419</v>
       </c>
       <c r="C5" t="s" s="17">
-        <v>1413</v>
+        <v>1420</v>
       </c>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
@@ -57805,10 +57860,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s" s="9">
-        <v>1414</v>
+        <v>1421</v>
       </c>
       <c r="C6" t="s" s="17">
-        <v>1415</v>
+        <v>1422</v>
       </c>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
@@ -57818,10 +57873,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s" s="9">
-        <v>1416</v>
+        <v>1423</v>
       </c>
       <c r="C7" t="s" s="17">
-        <v>1417</v>
+        <v>1424</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
@@ -57831,10 +57886,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s" s="9">
-        <v>1418</v>
+        <v>1425</v>
       </c>
       <c r="C8" t="s" s="17">
-        <v>1419</v>
+        <v>1426</v>
       </c>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
@@ -57844,10 +57899,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s" s="9">
-        <v>1420</v>
+        <v>1427</v>
       </c>
       <c r="C9" t="s" s="17">
-        <v>1421</v>
+        <v>1428</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>

</xml_diff>